<commit_message>
🏆 Expert Rankings Updated — 31 Jul 2026 18:50 IST
</commit_message>
<xml_diff>
--- a/output/MF_Expert_Rankings.xlsx
+++ b/output/MF_Expert_Rankings.xlsx
@@ -617,7 +617,7 @@
     <row r="1" ht="50" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>🏆  MF EXPERT RANKINGS  |  Generated: 30 Jul 2026 18:53</t>
+          <t>🏆  MF EXPERT RANKINGS  |  Generated: 31 Jul 2026 18:50</t>
         </is>
       </c>
     </row>
@@ -842,13 +842,13 @@
         </is>
       </c>
       <c r="C13" s="12" t="n">
-        <v>65.7</v>
+        <v>65.5</v>
       </c>
       <c r="D13" s="5" t="n">
-        <v>14.02</v>
+        <v>13.99</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>12.79</v>
+        <v>12.63</v>
       </c>
       <c r="F13" s="5" t="n">
         <v>0.84</v>
@@ -857,7 +857,7 @@
         <v>-22.15</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>8.77</v>
+        <v>8.65</v>
       </c>
     </row>
     <row r="14">
@@ -2081,22 +2081,22 @@
         </is>
       </c>
       <c r="C73" s="9" t="n">
-        <v>76.59999999999999</v>
+        <v>77.2</v>
       </c>
       <c r="D73" s="10" t="n">
-        <v>26.52</v>
+        <v>27.33</v>
       </c>
       <c r="E73" s="10" t="n">
-        <v>16.58</v>
+        <v>17.03</v>
       </c>
       <c r="F73" s="10" t="n">
-        <v>1.24</v>
+        <v>1.28</v>
       </c>
       <c r="G73" s="10" t="n">
         <v>-28.94</v>
       </c>
       <c r="H73" s="11" t="n">
-        <v>26.6</v>
+        <v>27.35</v>
       </c>
     </row>
     <row r="74">
@@ -2109,22 +2109,22 @@
         </is>
       </c>
       <c r="C74" s="12" t="n">
-        <v>75.2</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="D74" s="5" t="n">
-        <v>42.02</v>
+        <v>43.58</v>
       </c>
       <c r="E74" s="5" t="n">
-        <v>22.15</v>
+        <v>22.92</v>
       </c>
       <c r="F74" s="5" t="n">
-        <v>1.46</v>
+        <v>1.51</v>
       </c>
       <c r="G74" s="6" t="n">
         <v>-57.16</v>
       </c>
       <c r="H74" s="7" t="n">
-        <v>50.36</v>
+        <v>52.02</v>
       </c>
     </row>
     <row r="75">
@@ -2137,22 +2137,22 @@
         </is>
       </c>
       <c r="C75" s="9" t="n">
-        <v>75</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="D75" s="10" t="n">
-        <v>21.31</v>
+        <v>21.22</v>
       </c>
       <c r="E75" s="10" t="n">
-        <v>14.61</v>
+        <v>14.46</v>
       </c>
       <c r="F75" s="10" t="n">
-        <v>1.17</v>
+        <v>1.16</v>
       </c>
       <c r="G75" s="10" t="n">
         <v>-19.86</v>
       </c>
       <c r="H75" s="11" t="n">
-        <v>21.54</v>
+        <v>21.36</v>
       </c>
     </row>
     <row r="76">
@@ -2165,13 +2165,13 @@
         </is>
       </c>
       <c r="C76" s="12" t="n">
-        <v>74.59999999999999</v>
+        <v>74.7</v>
       </c>
       <c r="D76" s="5" t="n">
-        <v>22.41</v>
+        <v>22.55</v>
       </c>
       <c r="E76" s="5" t="n">
-        <v>17.78</v>
+        <v>17.82</v>
       </c>
       <c r="F76" s="5" t="n">
         <v>1.41</v>
@@ -2180,7 +2180,7 @@
         <v>-34.67</v>
       </c>
       <c r="H76" s="7" t="n">
-        <v>23.4</v>
+        <v>23.45</v>
       </c>
     </row>
     <row r="78">
@@ -2788,22 +2788,22 @@
         </is>
       </c>
       <c r="C107" s="3" t="n">
-        <v>77.2</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="D107" s="5" t="n">
-        <v>29.9</v>
+        <v>31.96</v>
       </c>
       <c r="E107" s="5" t="n">
-        <v>25.77</v>
+        <v>26.96</v>
       </c>
       <c r="F107" s="5" t="n">
-        <v>1.18</v>
+        <v>1.27</v>
       </c>
       <c r="G107" s="5" t="n">
         <v>-27.24</v>
       </c>
       <c r="H107" s="7" t="n">
-        <v>34.83</v>
+        <v>37.07</v>
       </c>
     </row>
     <row r="108">
@@ -2816,22 +2816,22 @@
         </is>
       </c>
       <c r="C108" s="9" t="n">
-        <v>74.3</v>
+        <v>75</v>
       </c>
       <c r="D108" s="10" t="n">
-        <v>23.6</v>
+        <v>24.49</v>
       </c>
       <c r="E108" s="10" t="n">
-        <v>13.18</v>
+        <v>13.62</v>
       </c>
       <c r="F108" s="10" t="n">
-        <v>0.87</v>
+        <v>0.91</v>
       </c>
       <c r="G108" s="13" t="n">
         <v>-45.32</v>
       </c>
       <c r="H108" s="11" t="n">
-        <v>26.15</v>
+        <v>27.02</v>
       </c>
     </row>
     <row r="109">
@@ -2844,13 +2844,13 @@
         </is>
       </c>
       <c r="C109" s="12" t="n">
-        <v>63.1</v>
+        <v>62.9</v>
       </c>
       <c r="D109" s="5" t="n">
-        <v>12.42</v>
+        <v>12.41</v>
       </c>
       <c r="E109" s="5" t="n">
-        <v>9.82</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="F109" s="5" t="n">
         <v>0.51</v>
@@ -2859,7 +2859,7 @@
         <v>-30.75</v>
       </c>
       <c r="H109" s="7" t="n">
-        <v>6.83</v>
+        <v>6.73</v>
       </c>
     </row>
     <row r="110">
@@ -2872,22 +2872,22 @@
         </is>
       </c>
       <c r="C110" s="9" t="n">
-        <v>61.6</v>
+        <v>61.9</v>
       </c>
       <c r="D110" s="10" t="n">
-        <v>11.48</v>
+        <v>11.67</v>
       </c>
       <c r="E110" s="10" t="n">
-        <v>9.4</v>
+        <v>9.33</v>
       </c>
       <c r="F110" s="10" t="n">
-        <v>0.43</v>
+        <v>0.44</v>
       </c>
       <c r="G110" s="10" t="n">
         <v>-29.85</v>
       </c>
       <c r="H110" s="11" t="n">
-        <v>5.64</v>
+        <v>5.74</v>
       </c>
     </row>
     <row r="111">
@@ -7299,67 +7299,67 @@
         </is>
       </c>
       <c r="C4" s="29" t="n">
-        <v>76.59999999999999</v>
+        <v>77.2</v>
       </c>
       <c r="D4" s="21" t="n">
-        <v>29.37</v>
+        <v>30.84</v>
       </c>
       <c r="E4" s="21" t="n">
-        <v>26.52</v>
+        <v>27.33</v>
       </c>
       <c r="F4" s="21" t="n">
-        <v>16.58</v>
+        <v>17.03</v>
       </c>
       <c r="G4" s="21" t="n">
-        <v>7.97</v>
+        <v>8.18</v>
       </c>
       <c r="H4" s="21" t="n">
-        <v>28.29</v>
+        <v>29.61</v>
       </c>
       <c r="I4" s="21" t="n">
-        <v>26.91</v>
+        <v>27.73</v>
       </c>
       <c r="J4" s="21" t="n">
-        <v>26.31</v>
+        <v>26.32</v>
       </c>
       <c r="K4" s="21" t="n">
-        <v>26.45</v>
+        <v>26.46</v>
       </c>
       <c r="L4" s="22" t="n">
-        <v>1.24</v>
+        <v>1.28</v>
       </c>
       <c r="M4" s="22" t="n">
-        <v>1.7</v>
+        <v>1.76</v>
       </c>
       <c r="N4" s="22" t="n">
-        <v>18.85</v>
+        <v>18.87</v>
       </c>
       <c r="O4" s="23" t="n">
         <v>-28.94</v>
       </c>
       <c r="P4" s="22" t="n">
-        <v>0.92</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="Q4" s="22" t="n">
         <v>-1.85</v>
       </c>
       <c r="R4" s="24" t="n">
-        <v>31.5</v>
+        <v>32.2</v>
       </c>
       <c r="S4" s="24" t="n">
         <v>31.2</v>
       </c>
       <c r="T4" s="21" t="n">
-        <v>26.6</v>
+        <v>27.35</v>
       </c>
       <c r="U4" s="25" t="n">
-        <v>0.296</v>
+        <v>0.297</v>
       </c>
       <c r="V4" s="25" t="n">
         <v>0.043</v>
       </c>
       <c r="W4" s="21" t="n">
-        <v>0.85</v>
+        <v>0.87</v>
       </c>
       <c r="X4" s="24" t="n">
         <v>87.59999999999999</v>
@@ -7368,7 +7368,7 @@
         <v>4.7</v>
       </c>
       <c r="Z4" s="19" t="n">
-        <v>21.552</v>
+        <v>21.9644</v>
       </c>
     </row>
     <row r="5">
@@ -7381,67 +7381,67 @@
         </is>
       </c>
       <c r="C5" s="16" t="n">
-        <v>75.2</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="D5" s="11" t="n">
-        <v>58.51</v>
+        <v>63.83</v>
       </c>
       <c r="E5" s="11" t="n">
-        <v>42.02</v>
+        <v>43.58</v>
       </c>
       <c r="F5" s="11" t="n">
-        <v>22.15</v>
+        <v>22.92</v>
       </c>
       <c r="G5" s="11" t="n">
-        <v>12.02</v>
+        <v>12.39</v>
       </c>
       <c r="H5" s="11" t="n">
-        <v>50.55</v>
+        <v>53.08</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>36.07</v>
+        <v>38.07</v>
       </c>
       <c r="J5" s="11" t="n">
-        <v>18.01</v>
+        <v>18.02</v>
       </c>
       <c r="K5" s="11" t="n">
         <v>10.63</v>
       </c>
       <c r="L5" s="10" t="n">
-        <v>1.46</v>
+        <v>1.51</v>
       </c>
       <c r="M5" s="10" t="n">
-        <v>2.06</v>
+        <v>2.14</v>
       </c>
       <c r="N5" s="10" t="n">
-        <v>34.45</v>
+        <v>34.48</v>
       </c>
       <c r="O5" s="13" t="n">
         <v>-57.16</v>
       </c>
       <c r="P5" s="10" t="n">
-        <v>0.74</v>
+        <v>0.76</v>
       </c>
       <c r="Q5" s="10" t="n">
-        <v>-3.38</v>
+        <v>-3.37</v>
       </c>
       <c r="R5" s="17" t="n">
-        <v>56.2</v>
+        <v>58.1</v>
       </c>
       <c r="S5" s="17" t="n">
         <v>27.6</v>
       </c>
       <c r="T5" s="11" t="n">
-        <v>50.36</v>
+        <v>52.02</v>
       </c>
       <c r="U5" s="18" t="n">
-        <v>0.527</v>
+        <v>0.528</v>
       </c>
       <c r="V5" s="18" t="n">
         <v>0.039</v>
       </c>
       <c r="W5" s="11" t="n">
-        <v>1.08</v>
+        <v>1.11</v>
       </c>
       <c r="X5" s="17" t="n">
         <v>55.5</v>
@@ -7450,7 +7450,7 @@
         <v>13.6</v>
       </c>
       <c r="Z5" s="8" t="n">
-        <v>52.5314</v>
+        <v>54.2816</v>
       </c>
     </row>
     <row r="6">
@@ -7463,25 +7463,25 @@
         </is>
       </c>
       <c r="C6" s="29" t="n">
-        <v>75</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="D6" s="21" t="n">
-        <v>21.7</v>
+        <v>21.16</v>
       </c>
       <c r="E6" s="21" t="n">
-        <v>21.31</v>
+        <v>21.22</v>
       </c>
       <c r="F6" s="21" t="n">
-        <v>14.61</v>
+        <v>14.46</v>
       </c>
       <c r="G6" s="21" t="n">
-        <v>9.890000000000001</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="H6" s="21" t="n">
-        <v>22.89</v>
+        <v>22.69</v>
       </c>
       <c r="I6" s="21" t="n">
-        <v>19.86</v>
+        <v>19.97</v>
       </c>
       <c r="J6" s="21" t="n">
         <v>16.27</v>
@@ -7490,13 +7490,13 @@
         <v>15.88</v>
       </c>
       <c r="L6" s="22" t="n">
-        <v>1.17</v>
+        <v>1.16</v>
       </c>
       <c r="M6" s="22" t="n">
-        <v>1.53</v>
+        <v>1.51</v>
       </c>
       <c r="N6" s="22" t="n">
-        <v>15.35</v>
+        <v>15.34</v>
       </c>
       <c r="O6" s="22" t="n">
         <v>-19.86</v>
@@ -7505,16 +7505,16 @@
         <v>1.07</v>
       </c>
       <c r="Q6" s="22" t="n">
-        <v>-1.45</v>
+        <v>-1.44</v>
       </c>
       <c r="R6" s="24" t="n">
-        <v>41.3</v>
+        <v>41.1</v>
       </c>
       <c r="S6" s="24" t="n">
         <v>52.1</v>
       </c>
       <c r="T6" s="21" t="n">
-        <v>21.54</v>
+        <v>21.36</v>
       </c>
       <c r="U6" s="25" t="n">
         <v>0.403</v>
@@ -7523,7 +7523,7 @@
         <v>0.122</v>
       </c>
       <c r="W6" s="21" t="n">
-        <v>0.95</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="X6" s="24" t="n">
         <v>83.7</v>
@@ -7532,7 +7532,7 @@
         <v>5.8</v>
       </c>
       <c r="Z6" s="19" t="n">
-        <v>25.6949</v>
+        <v>25.6362</v>
       </c>
     </row>
     <row r="7">
@@ -7545,25 +7545,25 @@
         </is>
       </c>
       <c r="C7" s="16" t="n">
-        <v>74.59999999999999</v>
+        <v>74.7</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>24.29</v>
+        <v>26.06</v>
       </c>
       <c r="E7" s="11" t="n">
-        <v>22.41</v>
+        <v>22.55</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>17.78</v>
+        <v>17.82</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>14.93</v>
+        <v>14.97</v>
       </c>
       <c r="H7" s="11" t="n">
-        <v>25.91</v>
+        <v>26.1</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>22.78</v>
+        <v>23.11</v>
       </c>
       <c r="J7" s="11" t="n">
         <v>12.92</v>
@@ -7575,10 +7575,10 @@
         <v>1.41</v>
       </c>
       <c r="M7" s="10" t="n">
-        <v>2</v>
+        <v>2.01</v>
       </c>
       <c r="N7" s="10" t="n">
-        <v>14.75</v>
+        <v>14.74</v>
       </c>
       <c r="O7" s="13" t="n">
         <v>-34.67</v>
@@ -7590,19 +7590,19 @@
         <v>-1.3</v>
       </c>
       <c r="R7" s="17" t="n">
-        <v>44.8</v>
+        <v>44.9</v>
       </c>
       <c r="S7" s="17" t="n">
         <v>52</v>
       </c>
       <c r="T7" s="11" t="n">
-        <v>23.4</v>
+        <v>23.45</v>
       </c>
       <c r="U7" s="18" t="n">
         <v>0.448</v>
       </c>
       <c r="V7" s="18" t="n">
-        <v>0.157</v>
+        <v>0.158</v>
       </c>
       <c r="W7" s="11" t="n">
         <v>1.13</v>
@@ -7614,7 +7614,7 @@
         <v>12.2</v>
       </c>
       <c r="Z7" s="8" t="n">
-        <v>42.7993</v>
+        <v>42.9379</v>
       </c>
     </row>
     <row r="8">
@@ -7710,28 +7710,28 @@
         <v>69.8</v>
       </c>
       <c r="D9" s="11" t="n">
-        <v>21.61</v>
+        <v>22.04</v>
       </c>
       <c r="E9" s="11" t="n">
-        <v>21.63</v>
+        <v>21.69</v>
       </c>
       <c r="F9" s="11" t="n">
-        <v>12.4</v>
+        <v>12.31</v>
       </c>
       <c r="G9" s="11" t="n">
-        <v>6.57</v>
+        <v>6.58</v>
       </c>
       <c r="H9" s="11" t="n">
-        <v>22.86</v>
+        <v>22.93</v>
       </c>
       <c r="I9" s="11" t="n">
-        <v>19.49</v>
+        <v>19.82</v>
       </c>
       <c r="J9" s="11" t="n">
         <v>15.02</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>16.77</v>
+        <v>16.78</v>
       </c>
       <c r="L9" s="10" t="n">
         <v>1</v>
@@ -7740,7 +7740,7 @@
         <v>1.31</v>
       </c>
       <c r="N9" s="10" t="n">
-        <v>19.16</v>
+        <v>19.14</v>
       </c>
       <c r="O9" s="13" t="n">
         <v>-30.84</v>
@@ -7758,7 +7758,7 @@
         <v>64.40000000000001</v>
       </c>
       <c r="T9" s="11" t="n">
-        <v>22.12</v>
+        <v>22.1</v>
       </c>
       <c r="U9" s="18" t="n">
         <v>0.477</v>
@@ -7776,7 +7776,7 @@
         <v>5.2</v>
       </c>
       <c r="Z9" s="8" t="n">
-        <v>18.91</v>
+        <v>18.94</v>
       </c>
     </row>
     <row r="10">
@@ -7789,25 +7789,25 @@
         </is>
       </c>
       <c r="C10" s="20" t="n">
-        <v>68.3</v>
+        <v>68.8</v>
       </c>
       <c r="D10" s="21" t="n">
-        <v>14.19</v>
+        <v>15.24</v>
       </c>
       <c r="E10" s="21" t="n">
-        <v>16.95</v>
+        <v>17.23</v>
       </c>
       <c r="F10" s="21" t="n">
-        <v>11.14</v>
+        <v>11.41</v>
       </c>
       <c r="G10" s="21" t="n">
-        <v>15.89</v>
+        <v>15.97</v>
       </c>
       <c r="H10" s="21" t="n">
-        <v>16.18</v>
+        <v>16.63</v>
       </c>
       <c r="I10" s="21" t="n">
-        <v>15.78</v>
+        <v>16.23</v>
       </c>
       <c r="J10" s="21" t="n">
         <v>16.65</v>
@@ -7816,37 +7816,37 @@
         <v>16.1</v>
       </c>
       <c r="L10" s="22" t="n">
-        <v>0.83</v>
+        <v>0.85</v>
       </c>
       <c r="M10" s="22" t="n">
-        <v>1.14</v>
+        <v>1.16</v>
       </c>
       <c r="N10" s="22" t="n">
-        <v>15.92</v>
+        <v>15.91</v>
       </c>
       <c r="O10" s="23" t="n">
         <v>-30.78</v>
       </c>
       <c r="P10" s="22" t="n">
-        <v>0.55</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="Q10" s="22" t="n">
         <v>-1.52</v>
       </c>
       <c r="R10" s="24" t="n">
-        <v>16.3</v>
+        <v>16.5</v>
       </c>
       <c r="S10" s="24" t="n">
         <v>15</v>
       </c>
       <c r="T10" s="21" t="n">
-        <v>18.68</v>
+        <v>18.93</v>
       </c>
       <c r="U10" s="25" t="n">
-        <v>0.116</v>
+        <v>0.117</v>
       </c>
       <c r="V10" s="25" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.01</v>
       </c>
       <c r="W10" s="21" t="n">
         <v>0.53</v>
@@ -7858,7 +7858,7 @@
         <v>11</v>
       </c>
       <c r="Z10" s="19" t="n">
-        <v>45.6025</v>
+        <v>45.9231</v>
       </c>
     </row>
     <row r="11">
@@ -7867,80 +7867,80 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>HSBC Global Emerging Market Fund - Growth Direct</t>
+          <t>DSP World Mining Overseas Equity Omni FoF - Direct Plan - Growth</t>
         </is>
       </c>
       <c r="C11" s="26" t="n">
-        <v>67.8</v>
+        <v>68.5</v>
       </c>
       <c r="D11" s="11" t="n">
-        <v>44.82</v>
+        <v>70.56</v>
       </c>
       <c r="E11" s="11" t="n">
-        <v>22.74</v>
+        <v>23.06</v>
       </c>
       <c r="F11" s="11" t="n">
-        <v>11.11</v>
+        <v>15.82</v>
       </c>
       <c r="G11" s="11" t="n">
-        <v>11.97</v>
+        <v>16.89</v>
       </c>
       <c r="H11" s="11" t="n">
-        <v>31.77</v>
+        <v>36.52</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>21.17</v>
+        <v>24.96</v>
       </c>
       <c r="J11" s="11" t="n">
-        <v>10.29</v>
+        <v>13.5</v>
       </c>
       <c r="K11" s="11" t="n">
-        <v>7.28</v>
+        <v>10.24</v>
       </c>
       <c r="L11" s="10" t="n">
-        <v>1.12</v>
+        <v>0.86</v>
       </c>
       <c r="M11" s="10" t="n">
-        <v>1.48</v>
+        <v>1.23</v>
       </c>
       <c r="N11" s="10" t="n">
-        <v>19.61</v>
+        <v>27.01</v>
       </c>
       <c r="O11" s="13" t="n">
-        <v>-34.59</v>
+        <v>-62.21</v>
       </c>
       <c r="P11" s="10" t="n">
-        <v>0.66</v>
+        <v>0.37</v>
       </c>
       <c r="Q11" s="10" t="n">
-        <v>-1.77</v>
+        <v>-2.64</v>
       </c>
       <c r="R11" s="17" t="n">
-        <v>71.40000000000001</v>
+        <v>64.3</v>
       </c>
       <c r="S11" s="17" t="n">
-        <v>73.5</v>
+        <v>67.5</v>
       </c>
       <c r="T11" s="11" t="n">
-        <v>22.89</v>
+        <v>23.66</v>
       </c>
       <c r="U11" s="18" t="n">
-        <v>0.681</v>
+        <v>0.59</v>
       </c>
       <c r="V11" s="18" t="n">
-        <v>0.218</v>
+        <v>0.079</v>
       </c>
       <c r="W11" s="11" t="n">
-        <v>1.04</v>
+        <v>0.68</v>
       </c>
       <c r="X11" s="17" t="n">
-        <v>67.2</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="Y11" s="17" t="n">
         <v>13.6</v>
       </c>
       <c r="Z11" s="8" t="n">
-        <v>35.2742</v>
+        <v>33.2789</v>
       </c>
     </row>
     <row r="12">
@@ -7949,80 +7949,80 @@
       </c>
       <c r="B12" s="19" t="inlineStr">
         <is>
-          <t>DSP World Mining Overseas Equity Omni FoF - Direct Plan - Growth</t>
+          <t>HSBC Global Emerging Market Fund - Growth Direct</t>
         </is>
       </c>
       <c r="C12" s="20" t="n">
-        <v>67.5</v>
+        <v>67.7</v>
       </c>
       <c r="D12" s="21" t="n">
-        <v>66.38</v>
+        <v>45</v>
       </c>
       <c r="E12" s="21" t="n">
-        <v>21.88</v>
+        <v>22.9</v>
       </c>
       <c r="F12" s="21" t="n">
-        <v>15.18</v>
+        <v>10.77</v>
       </c>
       <c r="G12" s="21" t="n">
-        <v>16.55</v>
+        <v>12.01</v>
       </c>
       <c r="H12" s="21" t="n">
-        <v>34.42</v>
+        <v>32</v>
       </c>
       <c r="I12" s="21" t="n">
-        <v>23.43</v>
+        <v>21.7</v>
       </c>
       <c r="J12" s="21" t="n">
-        <v>13.49</v>
+        <v>10.29</v>
       </c>
       <c r="K12" s="21" t="n">
-        <v>10.24</v>
+        <v>7.28</v>
       </c>
       <c r="L12" s="22" t="n">
-        <v>0.8100000000000001</v>
+        <v>1.13</v>
       </c>
       <c r="M12" s="22" t="n">
-        <v>1.16</v>
+        <v>1.49</v>
       </c>
       <c r="N12" s="22" t="n">
-        <v>26.98</v>
+        <v>19.6</v>
       </c>
       <c r="O12" s="23" t="n">
-        <v>-62.21</v>
+        <v>-34.59</v>
       </c>
       <c r="P12" s="22" t="n">
-        <v>0.35</v>
+        <v>0.66</v>
       </c>
       <c r="Q12" s="22" t="n">
-        <v>-2.64</v>
+        <v>-1.77</v>
       </c>
       <c r="R12" s="24" t="n">
-        <v>62.6</v>
+        <v>71.5</v>
       </c>
       <c r="S12" s="24" t="n">
-        <v>67.5</v>
+        <v>73.5</v>
       </c>
       <c r="T12" s="21" t="n">
-        <v>22.48</v>
+        <v>22.94</v>
       </c>
       <c r="U12" s="25" t="n">
-        <v>0.589</v>
+        <v>0.681</v>
       </c>
       <c r="V12" s="25" t="n">
-        <v>0.079</v>
+        <v>0.218</v>
       </c>
       <c r="W12" s="21" t="n">
-        <v>0.64</v>
+        <v>1.04</v>
       </c>
       <c r="X12" s="24" t="n">
-        <v>68.40000000000001</v>
+        <v>67.2</v>
       </c>
       <c r="Y12" s="24" t="n">
         <v>13.6</v>
       </c>
       <c r="Z12" s="19" t="n">
-        <v>32.3287</v>
+        <v>35.4116</v>
       </c>
     </row>
     <row r="13">
@@ -8031,80 +8031,80 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Principal Global Opportunities Fund-Direct Plan - Growth Option</t>
+          <t>Aditya Birla Sun Life International Equity Fund - Growth - Direct Plan</t>
         </is>
       </c>
       <c r="C13" s="26" t="n">
-        <v>66</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="D13" s="11" t="n">
-        <v>26.44</v>
+        <v>22.58</v>
       </c>
       <c r="E13" s="11" t="n">
-        <v>25.03</v>
+        <v>17.94</v>
       </c>
       <c r="F13" s="11" t="n">
-        <v>16.84</v>
+        <v>11.85</v>
       </c>
       <c r="G13" s="11" t="n">
-        <v>8.35</v>
+        <v>13.51</v>
       </c>
       <c r="H13" s="11" t="n">
-        <v>25.77</v>
+        <v>22.99</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>18.22</v>
+        <v>17.94</v>
       </c>
       <c r="J13" s="11" t="n">
-        <v>11.54</v>
+        <v>11.62</v>
       </c>
       <c r="K13" s="11" t="n">
-        <v>8.210000000000001</v>
+        <v>9.75</v>
       </c>
       <c r="L13" s="10" t="n">
-        <v>1.14</v>
+        <v>1.02</v>
       </c>
       <c r="M13" s="10" t="n">
-        <v>1.23</v>
+        <v>1.38</v>
       </c>
       <c r="N13" s="10" t="n">
-        <v>19.98</v>
+        <v>12.74</v>
       </c>
       <c r="O13" s="13" t="n">
-        <v>-37.39</v>
+        <v>-27.46</v>
       </c>
       <c r="P13" s="10" t="n">
-        <v>0.67</v>
+        <v>0.65</v>
       </c>
       <c r="Q13" s="10" t="n">
-        <v>-1.64</v>
+        <v>-1.19</v>
       </c>
       <c r="R13" s="17" t="n">
-        <v>12.9</v>
+        <v>18.1</v>
       </c>
       <c r="S13" s="17" t="n">
-        <v>27</v>
+        <v>20.1</v>
       </c>
       <c r="T13" s="11" t="n">
-        <v>22.45</v>
+        <v>17.75</v>
       </c>
       <c r="U13" s="18" t="n">
-        <v>0.233</v>
+        <v>0.172</v>
       </c>
       <c r="V13" s="18" t="n">
-        <v>0.063</v>
+        <v>0.032</v>
       </c>
       <c r="W13" s="11" t="n">
-        <v>0.09</v>
+        <v>0.54</v>
       </c>
       <c r="X13" s="17" t="n">
-        <v>68.2</v>
+        <v>84.5</v>
       </c>
       <c r="Y13" s="17" t="n">
-        <v>9</v>
+        <v>13.6</v>
       </c>
       <c r="Z13" s="8" t="n">
-        <v>49.2461</v>
+        <v>56.2156</v>
       </c>
     </row>
     <row r="14">
@@ -8113,80 +8113,80 @@
       </c>
       <c r="B14" s="19" t="inlineStr">
         <is>
-          <t>Aditya Birla Sun Life International Equity Fund - Growth - Direct Plan</t>
+          <t>Principal Global Opportunities Fund-Direct Plan - Growth Option</t>
         </is>
       </c>
       <c r="C14" s="20" t="n">
-        <v>65.5</v>
+        <v>66</v>
       </c>
       <c r="D14" s="21" t="n">
-        <v>21.42</v>
+        <v>26.44</v>
       </c>
       <c r="E14" s="21" t="n">
-        <v>17.15</v>
+        <v>25.03</v>
       </c>
       <c r="F14" s="21" t="n">
-        <v>11.36</v>
+        <v>16.84</v>
       </c>
       <c r="G14" s="21" t="n">
-        <v>13.29</v>
+        <v>8.35</v>
       </c>
       <c r="H14" s="21" t="n">
-        <v>21.61</v>
+        <v>25.77</v>
       </c>
       <c r="I14" s="21" t="n">
-        <v>16.91</v>
+        <v>18.22</v>
       </c>
       <c r="J14" s="21" t="n">
-        <v>11.61</v>
+        <v>11.54</v>
       </c>
       <c r="K14" s="21" t="n">
-        <v>9.75</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="L14" s="22" t="n">
-        <v>0.96</v>
+        <v>1.14</v>
       </c>
       <c r="M14" s="22" t="n">
-        <v>1.29</v>
+        <v>1.23</v>
       </c>
       <c r="N14" s="22" t="n">
-        <v>12.7</v>
+        <v>19.98</v>
       </c>
       <c r="O14" s="23" t="n">
-        <v>-27.46</v>
+        <v>-37.39</v>
       </c>
       <c r="P14" s="22" t="n">
-        <v>0.62</v>
+        <v>0.67</v>
       </c>
       <c r="Q14" s="22" t="n">
-        <v>-1.19</v>
+        <v>-1.64</v>
       </c>
       <c r="R14" s="24" t="n">
-        <v>17.5</v>
+        <v>12.9</v>
       </c>
       <c r="S14" s="24" t="n">
-        <v>20.1</v>
+        <v>27</v>
       </c>
       <c r="T14" s="21" t="n">
-        <v>16.98</v>
+        <v>22.45</v>
       </c>
       <c r="U14" s="25" t="n">
-        <v>0.171</v>
+        <v>0.233</v>
       </c>
       <c r="V14" s="25" t="n">
-        <v>0.032</v>
+        <v>0.063</v>
       </c>
       <c r="W14" s="21" t="n">
-        <v>0.51</v>
+        <v>0.09</v>
       </c>
       <c r="X14" s="24" t="n">
-        <v>84.5</v>
+        <v>68.2</v>
       </c>
       <c r="Y14" s="24" t="n">
-        <v>13.6</v>
+        <v>9</v>
       </c>
       <c r="Z14" s="19" t="n">
-        <v>55.0964</v>
+        <v>49.2461</v>
       </c>
     </row>
     <row r="15">
@@ -8199,25 +8199,25 @@
         </is>
       </c>
       <c r="C15" s="26" t="n">
-        <v>65.09999999999999</v>
+        <v>65.3</v>
       </c>
       <c r="D15" s="11" t="n">
-        <v>39.23</v>
+        <v>39.63</v>
       </c>
       <c r="E15" s="11" t="n">
-        <v>21.01</v>
+        <v>21.12</v>
       </c>
       <c r="F15" s="11" t="n">
-        <v>10.65</v>
+        <v>10.71</v>
       </c>
       <c r="G15" s="11" t="n">
-        <v>11.11</v>
+        <v>11.14</v>
       </c>
       <c r="H15" s="11" t="n">
-        <v>27.65</v>
+        <v>27.8</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>19.46</v>
+        <v>19.9</v>
       </c>
       <c r="J15" s="11" t="n">
         <v>9.98</v>
@@ -8229,10 +8229,10 @@
         <v>1.02</v>
       </c>
       <c r="M15" s="10" t="n">
-        <v>1.24</v>
+        <v>1.25</v>
       </c>
       <c r="N15" s="10" t="n">
-        <v>17.71</v>
+        <v>17.7</v>
       </c>
       <c r="O15" s="13" t="n">
         <v>-31.96</v>
@@ -8244,13 +8244,13 @@
         <v>-1.72</v>
       </c>
       <c r="R15" s="17" t="n">
-        <v>58.7</v>
+        <v>58.8</v>
       </c>
       <c r="S15" s="17" t="n">
         <v>69.7</v>
       </c>
       <c r="T15" s="11" t="n">
-        <v>18.74</v>
+        <v>18.77</v>
       </c>
       <c r="U15" s="18" t="n">
         <v>0.584</v>
@@ -8268,7 +8268,7 @@
         <v>13.6</v>
       </c>
       <c r="Z15" s="8" t="n">
-        <v>39.672</v>
+        <v>39.784</v>
       </c>
     </row>
     <row r="16">
@@ -8605,80 +8605,80 @@
       </c>
       <c r="B20" s="19" t="inlineStr">
         <is>
-          <t>ICICI Prudential Global Stable Equity Fund (FOF) - Direct - Growth</t>
+          <t>PGIM India Global Equity Opportunities Fund of Fund- Direct Plan - Growth</t>
         </is>
       </c>
       <c r="C20" s="20" t="n">
-        <v>62</v>
+        <v>62.2</v>
       </c>
       <c r="D20" s="21" t="n">
-        <v>23.51</v>
+        <v>10.1</v>
       </c>
       <c r="E20" s="21" t="n">
-        <v>13.91</v>
+        <v>15.28</v>
       </c>
       <c r="F20" s="21" t="n">
-        <v>10.9</v>
+        <v>6.3</v>
       </c>
       <c r="G20" s="21" t="n">
-        <v>10.39</v>
+        <v>14.73</v>
       </c>
       <c r="H20" s="21" t="n">
-        <v>17.72</v>
+        <v>12.74</v>
       </c>
       <c r="I20" s="21" t="n">
-        <v>14.51</v>
+        <v>13.56</v>
       </c>
       <c r="J20" s="21" t="n">
-        <v>10.43</v>
+        <v>17.81</v>
       </c>
       <c r="K20" s="21" t="n">
-        <v>9.67</v>
+        <v>16.51</v>
       </c>
       <c r="L20" s="22" t="n">
-        <v>0.84</v>
+        <v>0.62</v>
       </c>
       <c r="M20" s="22" t="n">
-        <v>1.17</v>
+        <v>0.85</v>
       </c>
       <c r="N20" s="22" t="n">
-        <v>11.75</v>
+        <v>21.04</v>
       </c>
       <c r="O20" s="23" t="n">
-        <v>-26.16</v>
+        <v>-43.42</v>
       </c>
       <c r="P20" s="22" t="n">
-        <v>0.53</v>
+        <v>0.35</v>
       </c>
       <c r="Q20" s="22" t="n">
-        <v>-1.08</v>
+        <v>-2.09</v>
       </c>
       <c r="R20" s="24" t="n">
-        <v>20.6</v>
+        <v>26.7</v>
       </c>
       <c r="S20" s="24" t="n">
-        <v>30.7</v>
+        <v>38.6</v>
       </c>
       <c r="T20" s="21" t="n">
-        <v>14.2</v>
+        <v>17.16</v>
       </c>
       <c r="U20" s="25" t="n">
-        <v>0.251</v>
+        <v>0.248</v>
       </c>
       <c r="V20" s="25" t="n">
-        <v>0.077</v>
+        <v>0.025</v>
       </c>
       <c r="W20" s="21" t="n">
-        <v>0.51</v>
+        <v>0.43</v>
       </c>
       <c r="X20" s="24" t="n">
-        <v>95.5</v>
+        <v>84.3</v>
       </c>
       <c r="Y20" s="24" t="n">
-        <v>12.9</v>
+        <v>10.4</v>
       </c>
       <c r="Z20" s="19" t="n">
-        <v>37.04</v>
+        <v>55.8</v>
       </c>
     </row>
     <row r="21">
@@ -8687,80 +8687,80 @@
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>Kotak US Equity Fund - Direct Plan - Growth option</t>
+          <t>ICICI Prudential Global Stable Equity Fund (FOF) - Direct - Growth</t>
         </is>
       </c>
       <c r="C21" s="26" t="n">
-        <v>60.5</v>
+        <v>61.2</v>
       </c>
       <c r="D21" s="11" t="n">
-        <v>17.12</v>
+        <v>21.44</v>
       </c>
       <c r="E21" s="11" t="n">
-        <v>13.33</v>
+        <v>13.45</v>
       </c>
       <c r="F21" s="11" t="n">
-        <v>11.68</v>
+        <v>10.63</v>
       </c>
       <c r="G21" s="11" t="n">
-        <v>6.17</v>
+        <v>10.26</v>
       </c>
       <c r="H21" s="11" t="n">
-        <v>15.3</v>
+        <v>16.85</v>
       </c>
       <c r="I21" s="11" t="n">
-        <v>13.95</v>
+        <v>14.15</v>
       </c>
       <c r="J21" s="11" t="n">
-        <v>11.32</v>
+        <v>10.43</v>
       </c>
       <c r="K21" s="11" t="n">
-        <v>12.25</v>
+        <v>9.67</v>
       </c>
       <c r="L21" s="10" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="M21" s="10" t="n">
-        <v>0.88</v>
+        <v>1.1</v>
       </c>
       <c r="N21" s="10" t="n">
-        <v>13.03</v>
-      </c>
-      <c r="O21" s="10" t="n">
-        <v>-22.42</v>
+        <v>11.77</v>
+      </c>
+      <c r="O21" s="13" t="n">
+        <v>-26.16</v>
       </c>
       <c r="P21" s="10" t="n">
-        <v>0.59</v>
+        <v>0.51</v>
       </c>
       <c r="Q21" s="10" t="n">
-        <v>-1.34</v>
+        <v>-1.12</v>
       </c>
       <c r="R21" s="17" t="n">
-        <v>7.2</v>
+        <v>20.2</v>
       </c>
       <c r="S21" s="17" t="n">
-        <v>-8.199999999999999</v>
+        <v>30.7</v>
       </c>
       <c r="T21" s="11" t="n">
-        <v>15.51</v>
+        <v>13.64</v>
       </c>
       <c r="U21" s="18" t="n">
-        <v>0.011</v>
+        <v>0.25</v>
       </c>
       <c r="V21" s="18" t="n">
-        <v>0</v>
+        <v>0.076</v>
       </c>
       <c r="W21" s="11" t="n">
-        <v>0.17</v>
+        <v>0.47</v>
       </c>
       <c r="X21" s="17" t="n">
-        <v>92.5</v>
+        <v>95.5</v>
       </c>
       <c r="Y21" s="17" t="n">
-        <v>5.1</v>
+        <v>12.9</v>
       </c>
       <c r="Z21" s="8" t="n">
-        <v>20.129</v>
+        <v>36.59</v>
       </c>
     </row>
     <row r="22">
@@ -8769,80 +8769,80 @@
       </c>
       <c r="B22" s="19" t="inlineStr">
         <is>
-          <t>Aditya Birla Sun Life International Equity Fund - Plan B - Growth - Direct Plan</t>
+          <t>Kotak US Equity Fund - Direct Plan - Growth option</t>
         </is>
       </c>
       <c r="C22" s="20" t="n">
-        <v>60.4</v>
+        <v>60.5</v>
       </c>
       <c r="D22" s="21" t="n">
-        <v>14.21</v>
+        <v>17.12</v>
       </c>
       <c r="E22" s="21" t="n">
-        <v>19.43</v>
+        <v>13.33</v>
       </c>
       <c r="F22" s="21" t="n">
-        <v>9.470000000000001</v>
+        <v>11.68</v>
       </c>
       <c r="G22" s="21" t="n">
-        <v>12.05</v>
+        <v>6.17</v>
       </c>
       <c r="H22" s="21" t="n">
-        <v>12.23</v>
+        <v>15.3</v>
       </c>
       <c r="I22" s="21" t="n">
-        <v>12.76</v>
+        <v>13.95</v>
       </c>
       <c r="J22" s="21" t="n">
-        <v>12.54</v>
+        <v>11.32</v>
       </c>
       <c r="K22" s="21" t="n">
-        <v>10.7</v>
+        <v>12.25</v>
       </c>
       <c r="L22" s="22" t="n">
-        <v>1.06</v>
+        <v>0.7</v>
       </c>
       <c r="M22" s="22" t="n">
-        <v>1.45</v>
+        <v>0.88</v>
       </c>
       <c r="N22" s="22" t="n">
-        <v>13.61</v>
-      </c>
-      <c r="O22" s="23" t="n">
-        <v>-36.39</v>
+        <v>13.03</v>
+      </c>
+      <c r="O22" s="22" t="n">
+        <v>-22.42</v>
       </c>
       <c r="P22" s="22" t="n">
-        <v>0.53</v>
+        <v>0.59</v>
       </c>
       <c r="Q22" s="22" t="n">
-        <v>-1.42</v>
+        <v>-1.34</v>
       </c>
       <c r="R22" s="24" t="n">
-        <v>63.7</v>
+        <v>7.2</v>
       </c>
       <c r="S22" s="24" t="n">
-        <v>90</v>
+        <v>-8.199999999999999</v>
       </c>
       <c r="T22" s="21" t="n">
-        <v>2.91</v>
+        <v>15.51</v>
       </c>
       <c r="U22" s="25" t="n">
-        <v>0.784</v>
+        <v>0.011</v>
       </c>
       <c r="V22" s="25" t="n">
-        <v>0.777</v>
-      </c>
-      <c r="W22" s="23" t="n">
-        <v>-0.22</v>
+        <v>0</v>
+      </c>
+      <c r="W22" s="21" t="n">
+        <v>0.17</v>
       </c>
       <c r="X22" s="24" t="n">
-        <v>73.7</v>
+        <v>92.5</v>
       </c>
       <c r="Y22" s="24" t="n">
-        <v>10.6</v>
+        <v>5.1</v>
       </c>
       <c r="Z22" s="19" t="n">
-        <v>30.2806</v>
+        <v>20.129</v>
       </c>
     </row>
     <row r="23">
@@ -8851,80 +8851,80 @@
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>PGIM India Global Equity Opportunities Fund of Fund- Direct Plan - Growth</t>
+          <t>Aditya Birla Sun Life International Equity Fund - Plan B - Growth - Direct Plan</t>
         </is>
       </c>
       <c r="C23" s="26" t="n">
-        <v>59.7</v>
+        <v>60.4</v>
       </c>
       <c r="D23" s="11" t="n">
-        <v>6.03</v>
+        <v>14.21</v>
       </c>
       <c r="E23" s="11" t="n">
-        <v>13.66</v>
+        <v>19.43</v>
       </c>
       <c r="F23" s="11" t="n">
-        <v>5.41</v>
+        <v>9.470000000000001</v>
       </c>
       <c r="G23" s="11" t="n">
-        <v>14.24</v>
+        <v>12.05</v>
       </c>
       <c r="H23" s="11" t="n">
-        <v>9.92</v>
+        <v>12.23</v>
       </c>
       <c r="I23" s="11" t="n">
-        <v>11.63</v>
+        <v>12.76</v>
       </c>
       <c r="J23" s="11" t="n">
-        <v>17.8</v>
+        <v>12.54</v>
       </c>
       <c r="K23" s="11" t="n">
-        <v>16.51</v>
+        <v>10.7</v>
       </c>
       <c r="L23" s="10" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="M23" s="10" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="N23" s="10" t="n">
+        <v>13.61</v>
+      </c>
+      <c r="O23" s="13" t="n">
+        <v>-36.39</v>
+      </c>
+      <c r="P23" s="10" t="n">
         <v>0.53</v>
       </c>
-      <c r="M23" s="10" t="n">
-        <v>0.73</v>
-      </c>
-      <c r="N23" s="10" t="n">
-        <v>20.9</v>
-      </c>
-      <c r="O23" s="13" t="n">
-        <v>-43.42</v>
-      </c>
-      <c r="P23" s="10" t="n">
-        <v>0.31</v>
-      </c>
       <c r="Q23" s="10" t="n">
-        <v>-2.09</v>
+        <v>-1.42</v>
       </c>
       <c r="R23" s="17" t="n">
-        <v>25.1</v>
+        <v>63.7</v>
       </c>
       <c r="S23" s="17" t="n">
-        <v>38.6</v>
+        <v>90</v>
       </c>
       <c r="T23" s="11" t="n">
-        <v>15.4</v>
+        <v>2.91</v>
       </c>
       <c r="U23" s="18" t="n">
-        <v>0.246</v>
+        <v>0.784</v>
       </c>
       <c r="V23" s="18" t="n">
-        <v>0.025</v>
-      </c>
-      <c r="W23" s="11" t="n">
-        <v>0.37</v>
+        <v>0.777</v>
+      </c>
+      <c r="W23" s="13" t="n">
+        <v>-0.22</v>
       </c>
       <c r="X23" s="17" t="n">
-        <v>84.3</v>
+        <v>73.7</v>
       </c>
       <c r="Y23" s="17" t="n">
-        <v>10.4</v>
+        <v>10.6</v>
       </c>
       <c r="Z23" s="8" t="n">
-        <v>53.48</v>
+        <v>30.2806</v>
       </c>
     </row>
     <row r="24">
@@ -9179,78 +9179,80 @@
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>PGIM India Global Select Real Estate Securities Fund of Fund - Direct Plan - Growth Option</t>
+          <t>DSP Global Clean Energy Overseas Equity Omni FoF Direct Plan - Growth</t>
         </is>
       </c>
       <c r="C27" s="26" t="n">
-        <v>56</v>
+        <v>56.8</v>
       </c>
       <c r="D27" s="11" t="n">
-        <v>27.39</v>
+        <v>40.29</v>
       </c>
       <c r="E27" s="11" t="n">
-        <v>16.08</v>
+        <v>15.63</v>
       </c>
       <c r="F27" s="11" t="n">
-        <v>6.61</v>
+        <v>12.35</v>
       </c>
       <c r="G27" s="11" t="n">
-        <v>3.25</v>
+        <v>9.58</v>
       </c>
       <c r="H27" s="11" t="n">
-        <v>20.08</v>
+        <v>26.7</v>
       </c>
       <c r="I27" s="11" t="n">
-        <v>15.15</v>
+        <v>18.95</v>
       </c>
       <c r="J27" s="11" t="n">
-        <v>9.25</v>
-      </c>
-      <c r="K27" s="13" t="n"/>
+        <v>7.81</v>
+      </c>
+      <c r="K27" s="11" t="n">
+        <v>4.48</v>
+      </c>
       <c r="L27" s="10" t="n">
-        <v>0.88</v>
+        <v>0.63</v>
       </c>
       <c r="M27" s="10" t="n">
-        <v>1.27</v>
+        <v>0.95</v>
       </c>
       <c r="N27" s="10" t="n">
-        <v>14.18</v>
+        <v>20.4</v>
       </c>
       <c r="O27" s="13" t="n">
-        <v>-27.4</v>
+        <v>-49.73</v>
       </c>
       <c r="P27" s="10" t="n">
-        <v>0.59</v>
+        <v>0.31</v>
       </c>
       <c r="Q27" s="10" t="n">
-        <v>-1.41</v>
+        <v>-2</v>
       </c>
       <c r="R27" s="17" t="n">
-        <v>13.5</v>
+        <v>48.1</v>
       </c>
       <c r="S27" s="17" t="n">
-        <v>8.1</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="T27" s="11" t="n">
-        <v>17.7</v>
+        <v>15.34</v>
       </c>
       <c r="U27" s="18" t="n">
-        <v>0.135</v>
+        <v>0.427</v>
       </c>
       <c r="V27" s="18" t="n">
-        <v>0.016</v>
+        <v>0.073</v>
       </c>
       <c r="W27" s="11" t="n">
-        <v>0.53</v>
+        <v>0.46</v>
       </c>
       <c r="X27" s="17" t="n">
-        <v>80.5</v>
+        <v>58.4</v>
       </c>
       <c r="Y27" s="17" t="n">
-        <v>4.6</v>
+        <v>13.6</v>
       </c>
       <c r="Z27" s="8" t="n">
-        <v>14.42</v>
+        <v>29.9851</v>
       </c>
     </row>
     <row r="28">
@@ -9259,80 +9261,78 @@
       </c>
       <c r="B28" s="19" t="inlineStr">
         <is>
-          <t>DSP Global Clean Energy Overseas Equity Omni FoF Direct Plan - Growth</t>
+          <t>PGIM India Global Select Real Estate Securities Fund of Fund - Direct Plan - Growth Option</t>
         </is>
       </c>
       <c r="C28" s="20" t="n">
-        <v>55.4</v>
+        <v>55.7</v>
       </c>
       <c r="D28" s="21" t="n">
-        <v>36.81</v>
+        <v>27.71</v>
       </c>
       <c r="E28" s="21" t="n">
-        <v>14.71</v>
+        <v>15.97</v>
       </c>
       <c r="F28" s="21" t="n">
-        <v>12.01</v>
+        <v>6.55</v>
       </c>
       <c r="G28" s="21" t="n">
-        <v>9.32</v>
+        <v>3.22</v>
       </c>
       <c r="H28" s="21" t="n">
-        <v>25.03</v>
+        <v>19.85</v>
       </c>
       <c r="I28" s="21" t="n">
-        <v>17.76</v>
+        <v>15.01</v>
       </c>
       <c r="J28" s="21" t="n">
-        <v>7.81</v>
-      </c>
-      <c r="K28" s="21" t="n">
-        <v>4.48</v>
-      </c>
+        <v>9.25</v>
+      </c>
+      <c r="K28" s="23" t="n"/>
       <c r="L28" s="22" t="n">
-        <v>0.59</v>
+        <v>0.87</v>
       </c>
       <c r="M28" s="22" t="n">
-        <v>0.87</v>
+        <v>1.25</v>
       </c>
       <c r="N28" s="22" t="n">
-        <v>20.36</v>
+        <v>14.17</v>
       </c>
       <c r="O28" s="23" t="n">
-        <v>-49.73</v>
+        <v>-27.4</v>
       </c>
       <c r="P28" s="22" t="n">
-        <v>0.3</v>
+        <v>0.58</v>
       </c>
       <c r="Q28" s="22" t="n">
-        <v>-2</v>
+        <v>-1.41</v>
       </c>
       <c r="R28" s="24" t="n">
-        <v>46.9</v>
+        <v>13.4</v>
       </c>
       <c r="S28" s="24" t="n">
-        <v>65.09999999999999</v>
+        <v>8.1</v>
       </c>
       <c r="T28" s="21" t="n">
-        <v>14.42</v>
+        <v>17.54</v>
       </c>
       <c r="U28" s="25" t="n">
-        <v>0.426</v>
+        <v>0.135</v>
       </c>
       <c r="V28" s="25" t="n">
-        <v>0.073</v>
+        <v>0.016</v>
       </c>
       <c r="W28" s="21" t="n">
-        <v>0.42</v>
+        <v>0.52</v>
       </c>
       <c r="X28" s="24" t="n">
-        <v>58.4</v>
+        <v>80.5</v>
       </c>
       <c r="Y28" s="24" t="n">
-        <v>13.6</v>
+        <v>4.6</v>
       </c>
       <c r="Z28" s="19" t="n">
-        <v>29.2763</v>
+        <v>14.38</v>
       </c>
     </row>
     <row r="29">
@@ -9341,85 +9341,83 @@
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>Invesco India - Invesco Global Consumer Trends Fund of Fund - Direct Plan - Growth</t>
+          <t>Mirae Asset Global Electric &amp; Autonomous Vehicles Equity Passive FOF - Direct Plan - Growth</t>
         </is>
       </c>
       <c r="C29" s="26" t="n">
-        <v>55.1</v>
+        <v>54.2</v>
       </c>
       <c r="D29" s="11" t="n">
-        <v>6.34</v>
+        <v>48.93</v>
       </c>
       <c r="E29" s="11" t="n">
-        <v>16.9</v>
+        <v>11.58</v>
       </c>
       <c r="F29" s="11" t="n">
-        <v>2.84</v>
+        <v>9.460000000000001</v>
       </c>
       <c r="G29" s="11" t="n">
-        <v>1.96</v>
+        <v>4.63</v>
       </c>
       <c r="H29" s="11" t="n">
-        <v>18.24</v>
+        <v>25.65</v>
       </c>
       <c r="I29" s="11" t="n">
-        <v>14.17</v>
+        <v>21.15</v>
       </c>
       <c r="J29" s="11" t="n">
-        <v>8.73</v>
-      </c>
-      <c r="K29" s="11" t="n">
-        <v>8.550000000000001</v>
-      </c>
+        <v>18.45</v>
+      </c>
+      <c r="K29" s="13" t="n"/>
       <c r="L29" s="10" t="n">
-        <v>0.62</v>
+        <v>0.36</v>
       </c>
       <c r="M29" s="10" t="n">
-        <v>0.84</v>
+        <v>0.48</v>
       </c>
       <c r="N29" s="10" t="n">
-        <v>29.81</v>
+        <v>28.11</v>
       </c>
       <c r="O29" s="13" t="n">
-        <v>-51.22</v>
+        <v>-30.41</v>
       </c>
       <c r="P29" s="10" t="n">
-        <v>0.33</v>
+        <v>0.38</v>
       </c>
       <c r="Q29" s="10" t="n">
-        <v>-3.28</v>
+        <v>-2.38</v>
       </c>
       <c r="R29" s="17" t="n">
-        <v>82.8</v>
+        <v>27.7</v>
       </c>
       <c r="S29" s="17" t="n">
-        <v>82</v>
+        <v>45.3</v>
       </c>
       <c r="T29" s="11" t="n">
-        <v>18.93</v>
+        <v>14.32</v>
       </c>
       <c r="U29" s="18" t="n">
-        <v>0.714</v>
+        <v>0.215</v>
       </c>
       <c r="V29" s="18" t="n">
-        <v>0.098</v>
+        <v>0.01</v>
       </c>
       <c r="W29" s="11" t="n">
-        <v>0.54</v>
+        <v>0.22</v>
       </c>
       <c r="X29" s="17" t="n">
-        <v>67.40000000000001</v>
+        <v>64.2</v>
       </c>
       <c r="Y29" s="17" t="n">
-        <v>5.6</v>
+        <v>3.9</v>
       </c>
       <c r="Z29" s="8" t="n">
-        <v>12.1571</v>
+        <v>15.877</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="19" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B30" s="19" t="inlineStr">
         <is>
@@ -9503,78 +9501,80 @@
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>Mirae Asset Global Electric &amp; Autonomous Vehicles Equity Passive FOF - Direct Plan - Growth</t>
+          <t>Invesco India - Invesco Global Consumer Trends Fund of Fund - Direct Plan - Growth</t>
         </is>
       </c>
       <c r="C31" s="26" t="n">
-        <v>52.9</v>
+        <v>52.8</v>
       </c>
       <c r="D31" s="11" t="n">
-        <v>43.9</v>
+        <v>3.2</v>
       </c>
       <c r="E31" s="11" t="n">
-        <v>10.52</v>
+        <v>15.39</v>
       </c>
       <c r="F31" s="11" t="n">
-        <v>8.84</v>
+        <v>2.28</v>
       </c>
       <c r="G31" s="11" t="n">
-        <v>4.33</v>
+        <v>1.57</v>
       </c>
       <c r="H31" s="11" t="n">
-        <v>23.66</v>
+        <v>15.53</v>
       </c>
       <c r="I31" s="11" t="n">
-        <v>19.63</v>
+        <v>12.96</v>
       </c>
       <c r="J31" s="11" t="n">
-        <v>18.42</v>
-      </c>
-      <c r="K31" s="13" t="n"/>
+        <v>8.710000000000001</v>
+      </c>
+      <c r="K31" s="11" t="n">
+        <v>8.539999999999999</v>
+      </c>
       <c r="L31" s="10" t="n">
-        <v>0.32</v>
+        <v>0.55</v>
       </c>
       <c r="M31" s="10" t="n">
-        <v>0.43</v>
+        <v>0.75</v>
       </c>
       <c r="N31" s="10" t="n">
-        <v>28.08</v>
+        <v>29.89</v>
       </c>
       <c r="O31" s="13" t="n">
-        <v>-30.41</v>
+        <v>-51.22</v>
       </c>
       <c r="P31" s="10" t="n">
-        <v>0.35</v>
+        <v>0.3</v>
       </c>
       <c r="Q31" s="10" t="n">
-        <v>-2.38</v>
+        <v>-3.32</v>
       </c>
       <c r="R31" s="17" t="n">
-        <v>26.6</v>
+        <v>79.5</v>
       </c>
       <c r="S31" s="17" t="n">
-        <v>45.3</v>
+        <v>82</v>
       </c>
       <c r="T31" s="11" t="n">
-        <v>13.24</v>
+        <v>17.13</v>
       </c>
       <c r="U31" s="18" t="n">
-        <v>0.213</v>
+        <v>0.712</v>
       </c>
       <c r="V31" s="18" t="n">
-        <v>0.01</v>
+        <v>0.096</v>
       </c>
       <c r="W31" s="11" t="n">
-        <v>0.19</v>
+        <v>0.48</v>
       </c>
       <c r="X31" s="17" t="n">
-        <v>64.2</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="Y31" s="17" t="n">
-        <v>3.9</v>
+        <v>5.6</v>
       </c>
       <c r="Z31" s="8" t="n">
-        <v>15.43</v>
+        <v>11.6926</v>
       </c>
     </row>
     <row r="32">
@@ -9587,66 +9587,66 @@
         </is>
       </c>
       <c r="C32" s="27" t="n">
-        <v>46</v>
+        <v>46.6</v>
       </c>
       <c r="D32" s="21" t="n">
-        <v>10.22</v>
+        <v>11.01</v>
       </c>
       <c r="E32" s="21" t="n">
-        <v>3.3</v>
+        <v>3.54</v>
       </c>
       <c r="F32" s="21" t="n">
-        <v>1.96</v>
+        <v>2.11</v>
       </c>
       <c r="G32" s="21" t="n">
-        <v>0.98</v>
+        <v>1.05</v>
       </c>
       <c r="H32" s="23" t="n"/>
       <c r="I32" s="23" t="n"/>
       <c r="J32" s="23" t="n"/>
       <c r="K32" s="23" t="n"/>
       <c r="L32" s="22" t="n">
-        <v>2.77</v>
+        <v>3.01</v>
       </c>
       <c r="M32" s="22" t="n">
-        <v>3.59</v>
+        <v>3.89</v>
       </c>
       <c r="N32" s="22" t="n">
-        <v>11.49</v>
+        <v>11.46</v>
       </c>
       <c r="O32" s="22" t="n">
         <v>-3.86</v>
       </c>
       <c r="P32" s="22" t="n">
-        <v>0.85</v>
+        <v>0.92</v>
       </c>
       <c r="Q32" s="22" t="n">
-        <v>-1.11</v>
+        <v>-1.08</v>
       </c>
       <c r="R32" s="24" t="n">
-        <v>10.3</v>
+        <v>11.7</v>
       </c>
       <c r="S32" s="24" t="n">
         <v>-27</v>
       </c>
       <c r="T32" s="21" t="n">
-        <v>37.36</v>
+        <v>39.91</v>
       </c>
       <c r="U32" s="25" t="n">
-        <v>0.029</v>
+        <v>0.03</v>
       </c>
       <c r="V32" s="25" t="n">
         <v>0.001</v>
       </c>
       <c r="W32" s="21" t="n">
-        <v>0.36</v>
+        <v>0.44</v>
       </c>
       <c r="X32" s="24" t="n"/>
       <c r="Y32" s="24" t="n">
         <v>0.3</v>
       </c>
       <c r="Z32" s="19" t="n">
-        <v>11.036</v>
+        <v>11.115</v>
       </c>
     </row>
     <row r="33">
@@ -9741,67 +9741,67 @@
         </is>
       </c>
       <c r="C34" s="27" t="n">
-        <v>45.1</v>
+        <v>43.5</v>
       </c>
       <c r="D34" s="21" t="n">
-        <v>14.56</v>
+        <v>10.05</v>
       </c>
       <c r="E34" s="21" t="n">
-        <v>10.09</v>
+        <v>9.18</v>
       </c>
       <c r="F34" s="21" t="n">
-        <v>4.22</v>
+        <v>3.72</v>
       </c>
       <c r="G34" s="21" t="n">
-        <v>2.4</v>
+        <v>2.15</v>
       </c>
       <c r="H34" s="21" t="n">
-        <v>13.65</v>
+        <v>11.95</v>
       </c>
       <c r="I34" s="21" t="n">
-        <v>8.9</v>
+        <v>8.06</v>
       </c>
       <c r="J34" s="21" t="n">
-        <v>4.33</v>
+        <v>4.32</v>
       </c>
       <c r="K34" s="21" t="n">
         <v>3</v>
       </c>
       <c r="L34" s="22" t="n">
-        <v>0.41</v>
+        <v>0.34</v>
       </c>
       <c r="M34" s="22" t="n">
-        <v>0.63</v>
+        <v>0.53</v>
       </c>
       <c r="N34" s="22" t="n">
-        <v>17.15</v>
+        <v>17.21</v>
       </c>
       <c r="O34" s="23" t="n">
         <v>-25.54</v>
       </c>
       <c r="P34" s="22" t="n">
-        <v>0.4</v>
+        <v>0.36</v>
       </c>
       <c r="Q34" s="22" t="n">
-        <v>-1.63</v>
+        <v>-1.66</v>
       </c>
       <c r="R34" s="24" t="n">
-        <v>30.3</v>
+        <v>29.3</v>
       </c>
       <c r="S34" s="24" t="n">
         <v>52.5</v>
       </c>
       <c r="T34" s="21" t="n">
-        <v>10.59</v>
+        <v>9.49</v>
       </c>
       <c r="U34" s="25" t="n">
-        <v>0.408</v>
+        <v>0.407</v>
       </c>
       <c r="V34" s="25" t="n">
-        <v>0.1</v>
+        <v>0.099</v>
       </c>
       <c r="W34" s="21" t="n">
-        <v>0.35</v>
+        <v>0.29</v>
       </c>
       <c r="X34" s="24" t="n">
         <v>63.4</v>
@@ -9810,7 +9810,7 @@
         <v>5.6</v>
       </c>
       <c r="Z34" s="19" t="n">
-        <v>12.6635</v>
+        <v>12.3528</v>
       </c>
     </row>
     <row r="35">
@@ -13178,25 +13178,25 @@
         </is>
       </c>
       <c r="C34" s="20" t="n">
-        <v>58.8</v>
+        <v>58.7</v>
       </c>
       <c r="D34" s="21" t="n">
-        <v>0.88</v>
+        <v>1.01</v>
       </c>
       <c r="E34" s="21" t="n">
-        <v>10.91</v>
+        <v>10.96</v>
       </c>
       <c r="F34" s="21" t="n">
-        <v>9.869999999999999</v>
+        <v>9.75</v>
       </c>
       <c r="G34" s="21" t="n">
-        <v>11.13</v>
+        <v>11.15</v>
       </c>
       <c r="H34" s="21" t="n">
-        <v>6.7</v>
+        <v>6.78</v>
       </c>
       <c r="I34" s="21" t="n">
-        <v>9.6</v>
+        <v>9.640000000000001</v>
       </c>
       <c r="J34" s="21" t="n">
         <v>14.75</v>
@@ -13208,10 +13208,10 @@
         <v>0.45</v>
       </c>
       <c r="M34" s="22" t="n">
-        <v>0.62</v>
+        <v>0.63</v>
       </c>
       <c r="N34" s="22" t="n">
-        <v>12.74</v>
+        <v>12.73</v>
       </c>
       <c r="O34" s="23" t="n">
         <v>-36.25</v>
@@ -13220,16 +13220,16 @@
         <v>0.3</v>
       </c>
       <c r="Q34" s="22" t="n">
-        <v>-1.3</v>
+        <v>-1.29</v>
       </c>
       <c r="R34" s="24" t="n">
-        <v>90.90000000000001</v>
+        <v>90.8</v>
       </c>
       <c r="S34" s="24" t="n">
         <v>95.59999999999999</v>
       </c>
       <c r="T34" s="21" t="n">
-        <v>3.47</v>
+        <v>3.43</v>
       </c>
       <c r="U34" s="25" t="n">
         <v>0.927</v>
@@ -13238,7 +13238,7 @@
         <v>0.927</v>
       </c>
       <c r="W34" s="21" t="n">
-        <v>0.78</v>
+        <v>0.77</v>
       </c>
       <c r="X34" s="24" t="n">
         <v>81.7</v>
@@ -13247,7 +13247,7 @@
         <v>13.6</v>
       </c>
       <c r="Z34" s="19" t="n">
-        <v>1139.1655</v>
+        <v>1140.7752</v>
       </c>
     </row>
     <row r="35">
@@ -18482,22 +18482,22 @@
         <v>73.09999999999999</v>
       </c>
       <c r="D46" s="21" t="n">
-        <v>7.08</v>
+        <v>6.91</v>
       </c>
       <c r="E46" s="21" t="n">
-        <v>16.12</v>
+        <v>16.23</v>
       </c>
       <c r="F46" s="21" t="n">
-        <v>13.71</v>
+        <v>13.4</v>
       </c>
       <c r="G46" s="21" t="n">
-        <v>14.34</v>
+        <v>14.37</v>
       </c>
       <c r="H46" s="21" t="n">
-        <v>11.42</v>
+        <v>11.59</v>
       </c>
       <c r="I46" s="21" t="n">
-        <v>14.2</v>
+        <v>14.33</v>
       </c>
       <c r="J46" s="21" t="n">
         <v>21.62</v>
@@ -18506,13 +18506,13 @@
         <v>21.47</v>
       </c>
       <c r="L46" s="22" t="n">
-        <v>0.83</v>
+        <v>0.84</v>
       </c>
       <c r="M46" s="22" t="n">
-        <v>1.07</v>
+        <v>1.08</v>
       </c>
       <c r="N46" s="22" t="n">
-        <v>13.34</v>
+        <v>13.33</v>
       </c>
       <c r="O46" s="23" t="n">
         <v>-31.87</v>
@@ -18524,13 +18524,13 @@
         <v>-1.32</v>
       </c>
       <c r="R46" s="24" t="n">
-        <v>88.5</v>
+        <v>88.59999999999999</v>
       </c>
       <c r="S46" s="24" t="n">
         <v>91.2</v>
       </c>
       <c r="T46" s="21" t="n">
-        <v>9</v>
+        <v>9.01</v>
       </c>
       <c r="U46" s="25" t="n">
         <v>0.886</v>
@@ -18548,7 +18548,7 @@
         <v>7.8</v>
       </c>
       <c r="Z46" s="19" t="n">
-        <v>38.27</v>
+        <v>38.38</v>
       </c>
     </row>
     <row r="47">
@@ -19295,25 +19295,25 @@
         </is>
       </c>
       <c r="C56" s="29" t="n">
-        <v>71</v>
+        <v>70.8</v>
       </c>
       <c r="D56" s="21" t="n">
-        <v>6.22</v>
+        <v>6.01</v>
       </c>
       <c r="E56" s="21" t="n">
-        <v>14.53</v>
+        <v>14.52</v>
       </c>
       <c r="F56" s="21" t="n">
-        <v>15.04</v>
+        <v>14.8</v>
       </c>
       <c r="G56" s="21" t="n">
-        <v>15.23</v>
+        <v>15.22</v>
       </c>
       <c r="H56" s="21" t="n">
-        <v>10.97</v>
+        <v>10.92</v>
       </c>
       <c r="I56" s="21" t="n">
-        <v>14.31</v>
+        <v>14.25</v>
       </c>
       <c r="J56" s="21" t="n">
         <v>19.5</v>
@@ -19328,7 +19328,7 @@
         <v>0.89</v>
       </c>
       <c r="N56" s="22" t="n">
-        <v>12.87</v>
+        <v>12.86</v>
       </c>
       <c r="O56" s="23" t="n">
         <v>-36.43</v>
@@ -19337,16 +19337,16 @@
         <v>0.4</v>
       </c>
       <c r="Q56" s="22" t="n">
-        <v>-1.34</v>
+        <v>-1.33</v>
       </c>
       <c r="R56" s="24" t="n">
-        <v>86.40000000000001</v>
+        <v>86.2</v>
       </c>
       <c r="S56" s="24" t="n">
         <v>91.59999999999999</v>
       </c>
       <c r="T56" s="21" t="n">
-        <v>7.31</v>
+        <v>7.2</v>
       </c>
       <c r="U56" s="25" t="n">
         <v>0.895</v>
@@ -19355,7 +19355,7 @@
         <v>0.837</v>
       </c>
       <c r="W56" s="21" t="n">
-        <v>1.14</v>
+        <v>1.12</v>
       </c>
       <c r="X56" s="24" t="n">
         <v>89.5</v>
@@ -19364,12 +19364,12 @@
         <v>13.6</v>
       </c>
       <c r="Z56" s="19" t="n">
-        <v>717.9623</v>
+        <v>717.6357</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="8" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B57" s="8" t="inlineStr">
         <is>
@@ -34392,65 +34392,65 @@
         </is>
       </c>
       <c r="C3" s="16" t="n">
-        <v>77.2</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="D3" s="11" t="n">
-        <v>37.21</v>
+        <v>43.35</v>
       </c>
       <c r="E3" s="11" t="n">
-        <v>29.9</v>
+        <v>31.96</v>
       </c>
       <c r="F3" s="11" t="n">
-        <v>25.77</v>
+        <v>26.96</v>
       </c>
       <c r="G3" s="11" t="n">
-        <v>12.15</v>
+        <v>12.68</v>
       </c>
       <c r="H3" s="11" t="n">
-        <v>34.07</v>
+        <v>37.55</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>34.95</v>
+        <v>37.61</v>
       </c>
       <c r="J3" s="11" t="n">
-        <v>37.88</v>
+        <v>37.93</v>
       </c>
       <c r="K3" s="13" t="n"/>
       <c r="L3" s="10" t="n">
-        <v>1.18</v>
+        <v>1.27</v>
       </c>
       <c r="M3" s="10" t="n">
-        <v>1.61</v>
+        <v>1.74</v>
       </c>
       <c r="N3" s="10" t="n">
-        <v>25.57</v>
+        <v>25.71</v>
       </c>
       <c r="O3" s="13" t="n">
         <v>-27.24</v>
       </c>
       <c r="P3" s="10" t="n">
-        <v>1.1</v>
+        <v>1.17</v>
       </c>
       <c r="Q3" s="10" t="n">
         <v>-2.53</v>
       </c>
       <c r="R3" s="17" t="n">
-        <v>29.2</v>
+        <v>31.1</v>
       </c>
       <c r="S3" s="17" t="n">
         <v>15.5</v>
       </c>
       <c r="T3" s="11" t="n">
-        <v>34.83</v>
+        <v>37.07</v>
       </c>
       <c r="U3" s="18" t="n">
-        <v>0.182</v>
+        <v>0.184</v>
       </c>
       <c r="V3" s="18" t="n">
         <v>0.008999999999999999</v>
       </c>
       <c r="W3" s="11" t="n">
-        <v>0.86</v>
+        <v>0.91</v>
       </c>
       <c r="X3" s="17" t="n">
         <v>99.3</v>
@@ -34459,7 +34459,7 @@
         <v>3.9</v>
       </c>
       <c r="Z3" s="8" t="n">
-        <v>31.475</v>
+        <v>33.002</v>
       </c>
     </row>
     <row r="4">
@@ -34472,67 +34472,67 @@
         </is>
       </c>
       <c r="C4" s="29" t="n">
-        <v>74.3</v>
+        <v>75</v>
       </c>
       <c r="D4" s="21" t="n">
-        <v>16.32</v>
+        <v>19.01</v>
       </c>
       <c r="E4" s="21" t="n">
-        <v>23.6</v>
+        <v>24.49</v>
       </c>
       <c r="F4" s="21" t="n">
-        <v>13.18</v>
+        <v>13.62</v>
       </c>
       <c r="G4" s="21" t="n">
-        <v>14.77</v>
+        <v>15.02</v>
       </c>
       <c r="H4" s="21" t="n">
-        <v>23.56</v>
+        <v>25.05</v>
       </c>
       <c r="I4" s="21" t="n">
-        <v>22.69</v>
+        <v>23.94</v>
       </c>
       <c r="J4" s="21" t="n">
-        <v>22.88</v>
+        <v>22.89</v>
       </c>
       <c r="K4" s="21" t="n">
-        <v>18.4</v>
+        <v>18.41</v>
       </c>
       <c r="L4" s="22" t="n">
-        <v>0.87</v>
+        <v>0.91</v>
       </c>
       <c r="M4" s="22" t="n">
-        <v>1.17</v>
+        <v>1.22</v>
       </c>
       <c r="N4" s="22" t="n">
-        <v>27.86</v>
+        <v>27.87</v>
       </c>
       <c r="O4" s="23" t="n">
         <v>-45.32</v>
       </c>
       <c r="P4" s="22" t="n">
-        <v>0.52</v>
+        <v>0.54</v>
       </c>
       <c r="Q4" s="22" t="n">
         <v>-2.89</v>
       </c>
       <c r="R4" s="24" t="n">
-        <v>81.59999999999999</v>
+        <v>83.09999999999999</v>
       </c>
       <c r="S4" s="24" t="n">
         <v>77.09999999999999</v>
       </c>
       <c r="T4" s="21" t="n">
-        <v>26.15</v>
+        <v>27.02</v>
       </c>
       <c r="U4" s="25" t="n">
-        <v>0.572</v>
+        <v>0.573</v>
       </c>
       <c r="V4" s="25" t="n">
         <v>0.076</v>
       </c>
       <c r="W4" s="21" t="n">
-        <v>0.75</v>
+        <v>0.77</v>
       </c>
       <c r="X4" s="24" t="n">
         <v>75.40000000000001</v>
@@ -34541,7 +34541,7 @@
         <v>6.4</v>
       </c>
       <c r="Z4" s="19" t="n">
-        <v>36.7405</v>
+        <v>37.5389</v>
       </c>
     </row>
     <row r="5">
@@ -34554,25 +34554,25 @@
         </is>
       </c>
       <c r="C5" s="26" t="n">
-        <v>63.1</v>
+        <v>62.9</v>
       </c>
       <c r="D5" s="13" t="n">
-        <v>-4.98</v>
+        <v>-5.1</v>
       </c>
       <c r="E5" s="11" t="n">
-        <v>12.42</v>
+        <v>12.41</v>
       </c>
       <c r="F5" s="11" t="n">
-        <v>9.82</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="G5" s="11" t="n">
         <v>16.19</v>
       </c>
       <c r="H5" s="11" t="n">
-        <v>3.31</v>
+        <v>3.29</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>9.67</v>
+        <v>9.65</v>
       </c>
       <c r="J5" s="11" t="n">
         <v>19.24</v>
@@ -34584,10 +34584,10 @@
         <v>0.51</v>
       </c>
       <c r="M5" s="10" t="n">
-        <v>0.76</v>
+        <v>0.75</v>
       </c>
       <c r="N5" s="10" t="n">
-        <v>15.02</v>
+        <v>15.01</v>
       </c>
       <c r="O5" s="13" t="n">
         <v>-30.75</v>
@@ -34599,13 +34599,13 @@
         <v>-1.49</v>
       </c>
       <c r="R5" s="17" t="n">
-        <v>78.2</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="S5" s="17" t="n">
         <v>89.8</v>
       </c>
       <c r="T5" s="11" t="n">
-        <v>6.83</v>
+        <v>6.73</v>
       </c>
       <c r="U5" s="18" t="n">
         <v>0.759</v>
@@ -34614,7 +34614,7 @@
         <v>0.447</v>
       </c>
       <c r="W5" s="11" t="n">
-        <v>0.39</v>
+        <v>0.38</v>
       </c>
       <c r="X5" s="17" t="n">
         <v>76.7</v>
@@ -34623,7 +34623,7 @@
         <v>13.6</v>
       </c>
       <c r="Z5" s="8" t="n">
-        <v>534.0788</v>
+        <v>533.9653</v>
       </c>
     </row>
     <row r="6">
@@ -34636,25 +34636,25 @@
         </is>
       </c>
       <c r="C6" s="20" t="n">
-        <v>61.6</v>
+        <v>61.9</v>
       </c>
       <c r="D6" s="23" t="n">
-        <v>-3.56</v>
+        <v>-3.26</v>
       </c>
       <c r="E6" s="21" t="n">
-        <v>11.48</v>
+        <v>11.67</v>
       </c>
       <c r="F6" s="21" t="n">
-        <v>9.4</v>
+        <v>9.33</v>
       </c>
       <c r="G6" s="21" t="n">
-        <v>16.64</v>
+        <v>16.7</v>
       </c>
       <c r="H6" s="21" t="n">
-        <v>4.81</v>
+        <v>5.12</v>
       </c>
       <c r="I6" s="21" t="n">
-        <v>8.43</v>
+        <v>8.59</v>
       </c>
       <c r="J6" s="21" t="n">
         <v>20.6</v>
@@ -34663,40 +34663,40 @@
         <v>18.51</v>
       </c>
       <c r="L6" s="22" t="n">
-        <v>0.43</v>
+        <v>0.44</v>
       </c>
       <c r="M6" s="22" t="n">
-        <v>0.63</v>
+        <v>0.65</v>
       </c>
       <c r="N6" s="22" t="n">
-        <v>15.28</v>
+        <v>15.27</v>
       </c>
       <c r="O6" s="23" t="n">
         <v>-29.85</v>
       </c>
       <c r="P6" s="22" t="n">
-        <v>0.38</v>
+        <v>0.39</v>
       </c>
       <c r="Q6" s="22" t="n">
         <v>-1.5</v>
       </c>
       <c r="R6" s="24" t="n">
-        <v>79.5</v>
+        <v>79.7</v>
       </c>
       <c r="S6" s="24" t="n">
         <v>90.90000000000001</v>
       </c>
       <c r="T6" s="21" t="n">
-        <v>5.64</v>
+        <v>5.74</v>
       </c>
       <c r="U6" s="25" t="n">
-        <v>0.794</v>
+        <v>0.795</v>
       </c>
       <c r="V6" s="25" t="n">
         <v>0.467</v>
       </c>
       <c r="W6" s="21" t="n">
-        <v>0.32</v>
+        <v>0.33</v>
       </c>
       <c r="X6" s="24" t="n">
         <v>78.2</v>
@@ -34705,7 +34705,7 @@
         <v>13.5</v>
       </c>
       <c r="Z6" s="19" t="n">
-        <v>233.1691</v>
+        <v>234.3394</v>
       </c>
     </row>
     <row r="7">
@@ -34800,25 +34800,25 @@
         </is>
       </c>
       <c r="C8" s="20" t="n">
-        <v>57.1</v>
+        <v>56.7</v>
       </c>
       <c r="D8" s="23" t="n">
-        <v>-5.64</v>
+        <v>-6.07</v>
       </c>
       <c r="E8" s="21" t="n">
-        <v>9.380000000000001</v>
+        <v>9.289999999999999</v>
       </c>
       <c r="F8" s="21" t="n">
-        <v>6.57</v>
+        <v>6.33</v>
       </c>
       <c r="G8" s="21" t="n">
-        <v>17.39</v>
+        <v>17.36</v>
       </c>
       <c r="H8" s="21" t="n">
-        <v>1.74</v>
+        <v>1.59</v>
       </c>
       <c r="I8" s="21" t="n">
-        <v>5.42</v>
+        <v>5.28</v>
       </c>
       <c r="J8" s="21" t="n">
         <v>22.85</v>
@@ -34830,37 +34830,37 @@
         <v>0.28</v>
       </c>
       <c r="M8" s="22" t="n">
-        <v>0.43</v>
+        <v>0.42</v>
       </c>
       <c r="N8" s="22" t="n">
-        <v>16.96</v>
+        <v>16.95</v>
       </c>
       <c r="O8" s="23" t="n">
         <v>-35.09</v>
       </c>
       <c r="P8" s="22" t="n">
-        <v>0.27</v>
+        <v>0.26</v>
       </c>
       <c r="Q8" s="22" t="n">
         <v>-1.62</v>
       </c>
       <c r="R8" s="24" t="n">
-        <v>91.7</v>
+        <v>91.3</v>
       </c>
       <c r="S8" s="24" t="n">
         <v>96.40000000000001</v>
       </c>
       <c r="T8" s="21" t="n">
-        <v>3.19</v>
+        <v>3.02</v>
       </c>
       <c r="U8" s="25" t="n">
-        <v>0.867</v>
+        <v>0.866</v>
       </c>
       <c r="V8" s="25" t="n">
-        <v>0.457</v>
+        <v>0.456</v>
       </c>
       <c r="W8" s="21" t="n">
-        <v>0.16</v>
+        <v>0.14</v>
       </c>
       <c r="X8" s="24" t="n">
         <v>72.3</v>
@@ -34869,7 +34869,7 @@
         <v>13.6</v>
       </c>
       <c r="Z8" s="19" t="n">
-        <v>205.76</v>
+        <v>205.28</v>
       </c>
     </row>
     <row r="9">
@@ -35046,65 +35046,65 @@
         </is>
       </c>
       <c r="C11" s="28" t="n">
-        <v>47.2</v>
+        <v>48.4</v>
       </c>
       <c r="D11" s="11" t="n">
-        <v>8.210000000000001</v>
+        <v>9.09</v>
       </c>
       <c r="E11" s="11" t="n">
-        <v>8.59</v>
+        <v>9.09</v>
       </c>
       <c r="F11" s="11" t="n">
-        <v>5.07</v>
+        <v>5.36</v>
       </c>
       <c r="G11" s="11" t="n">
-        <v>2.5</v>
+        <v>2.64</v>
       </c>
       <c r="H11" s="11" t="n">
-        <v>9.5</v>
+        <v>10.64</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>9.5</v>
+        <v>10.64</v>
       </c>
       <c r="J11" s="11" t="n">
-        <v>5.13</v>
+        <v>5.15</v>
       </c>
       <c r="K11" s="13" t="n"/>
       <c r="L11" s="10" t="n">
-        <v>0.4</v>
+        <v>0.45</v>
       </c>
       <c r="M11" s="10" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.62</v>
       </c>
       <c r="N11" s="10" t="n">
-        <v>15.09</v>
+        <v>15.1</v>
       </c>
       <c r="O11" s="13" t="n">
         <v>-26.24</v>
       </c>
       <c r="P11" s="10" t="n">
-        <v>0.33</v>
+        <v>0.35</v>
       </c>
       <c r="Q11" s="10" t="n">
         <v>-1.57</v>
       </c>
       <c r="R11" s="17" t="n">
-        <v>68.5</v>
+        <v>69.5</v>
       </c>
       <c r="S11" s="17" t="n">
         <v>85</v>
       </c>
       <c r="T11" s="11" t="n">
-        <v>8.48</v>
+        <v>9.01</v>
       </c>
       <c r="U11" s="18" t="n">
         <v>0.717</v>
       </c>
       <c r="V11" s="18" t="n">
-        <v>0.432</v>
+        <v>0.431</v>
       </c>
       <c r="W11" s="11" t="n">
-        <v>0.55</v>
+        <v>0.59</v>
       </c>
       <c r="X11" s="17" t="n">
         <v>86.3</v>
@@ -35113,7 +35113,7 @@
         <v>2.4</v>
       </c>
       <c r="Z11" s="8" t="n">
-        <v>12.8537</v>
+        <v>13.03</v>
       </c>
     </row>
     <row r="12">
@@ -35438,25 +35438,25 @@
         </is>
       </c>
       <c r="C16" s="27" t="n">
-        <v>28.6</v>
+        <v>28.7</v>
       </c>
       <c r="D16" s="23" t="n">
-        <v>-6.1</v>
+        <v>-5.94</v>
       </c>
       <c r="E16" s="21" t="n">
-        <v>2.72</v>
+        <v>2.81</v>
       </c>
       <c r="F16" s="21" t="n">
-        <v>1.62</v>
+        <v>1.68</v>
       </c>
       <c r="G16" s="21" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.83</v>
       </c>
       <c r="H16" s="23" t="n">
-        <v>-2.08</v>
+        <v>-1.87</v>
       </c>
       <c r="I16" s="23" t="n">
-        <v>-2.08</v>
+        <v>-1.87</v>
       </c>
       <c r="J16" s="23" t="n">
         <v>-2.97</v>
@@ -35466,10 +35466,10 @@
         <v>-0.08</v>
       </c>
       <c r="M16" s="22" t="n">
-        <v>-0.12</v>
+        <v>-0.11</v>
       </c>
       <c r="N16" s="22" t="n">
-        <v>17.22</v>
+        <v>17.21</v>
       </c>
       <c r="O16" s="23" t="n">
         <v>-28.59</v>
@@ -35487,7 +35487,7 @@
         <v>95.90000000000001</v>
       </c>
       <c r="T16" s="21" t="n">
-        <v>0.61</v>
+        <v>0.62</v>
       </c>
       <c r="U16" s="25" t="n">
         <v>0.86</v>
@@ -35505,7 +35505,7 @@
         <v>2.4</v>
       </c>
       <c r="Z16" s="19" t="n">
-        <v>10.859</v>
+        <v>10.887</v>
       </c>
     </row>
   </sheetData>
@@ -42188,25 +42188,25 @@
         </is>
       </c>
       <c r="C10" s="20" t="n">
-        <v>62.3</v>
+        <v>61.9</v>
       </c>
       <c r="D10" s="21" t="n">
-        <v>6.81</v>
+        <v>6.44</v>
       </c>
       <c r="E10" s="21" t="n">
-        <v>12.93</v>
+        <v>12.87</v>
       </c>
       <c r="F10" s="21" t="n">
-        <v>11.91</v>
+        <v>11.71</v>
       </c>
       <c r="G10" s="21" t="n">
-        <v>12.06</v>
+        <v>12.04</v>
       </c>
       <c r="H10" s="21" t="n">
-        <v>9.539999999999999</v>
+        <v>9.41</v>
       </c>
       <c r="I10" s="21" t="n">
-        <v>11.9</v>
+        <v>11.82</v>
       </c>
       <c r="J10" s="21" t="n">
         <v>12.78</v>
@@ -42218,7 +42218,7 @@
         <v>0.68</v>
       </c>
       <c r="M10" s="22" t="n">
-        <v>0.86</v>
+        <v>0.85</v>
       </c>
       <c r="N10" s="22" t="n">
         <v>11.4</v>
@@ -42227,28 +42227,28 @@
         <v>-31.06</v>
       </c>
       <c r="P10" s="22" t="n">
-        <v>0.42</v>
+        <v>0.41</v>
       </c>
       <c r="Q10" s="22" t="n">
         <v>-1.11</v>
       </c>
       <c r="R10" s="24" t="n">
-        <v>67.90000000000001</v>
+        <v>67.7</v>
       </c>
       <c r="S10" s="24" t="n">
         <v>84.5</v>
       </c>
       <c r="T10" s="21" t="n">
-        <v>7.36</v>
+        <v>7.21</v>
       </c>
       <c r="U10" s="25" t="n">
-        <v>0.784</v>
+        <v>0.783</v>
       </c>
       <c r="V10" s="25" t="n">
         <v>0.829</v>
       </c>
       <c r="W10" s="21" t="n">
-        <v>0.97</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="X10" s="24" t="n">
         <v>84.3</v>
@@ -42257,7 +42257,7 @@
         <v>12.2</v>
       </c>
       <c r="Z10" s="19" t="n">
-        <v>44.955</v>
+        <v>44.8806</v>
       </c>
     </row>
     <row r="11">
@@ -42516,25 +42516,25 @@
         </is>
       </c>
       <c r="C14" s="20" t="n">
-        <v>60.9</v>
+        <v>60.7</v>
       </c>
       <c r="D14" s="21" t="n">
-        <v>4.6</v>
+        <v>4.41</v>
       </c>
       <c r="E14" s="21" t="n">
-        <v>11.87</v>
+        <v>11.86</v>
       </c>
       <c r="F14" s="21" t="n">
-        <v>10.83</v>
+        <v>10.73</v>
       </c>
       <c r="G14" s="21" t="n">
-        <v>10.71</v>
+        <v>10.7</v>
       </c>
       <c r="H14" s="21" t="n">
-        <v>8.619999999999999</v>
+        <v>8.58</v>
       </c>
       <c r="I14" s="21" t="n">
-        <v>10.8</v>
+        <v>10.78</v>
       </c>
       <c r="J14" s="21" t="n">
         <v>11.06</v>
@@ -42549,7 +42549,7 @@
         <v>0.87</v>
       </c>
       <c r="N14" s="22" t="n">
-        <v>9.039999999999999</v>
+        <v>9.029999999999999</v>
       </c>
       <c r="O14" s="22" t="n">
         <v>-17.3</v>
@@ -42558,25 +42558,25 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="Q14" s="22" t="n">
-        <v>-0.9399999999999999</v>
+        <v>-0.93</v>
       </c>
       <c r="R14" s="24" t="n">
-        <v>46</v>
+        <v>45.9</v>
       </c>
       <c r="S14" s="24" t="n">
         <v>70.7</v>
       </c>
       <c r="T14" s="21" t="n">
-        <v>7.4</v>
+        <v>7.31</v>
       </c>
       <c r="U14" s="25" t="n">
         <v>0.614</v>
       </c>
       <c r="V14" s="25" t="n">
-        <v>0.767</v>
+        <v>0.766</v>
       </c>
       <c r="W14" s="21" t="n">
-        <v>0.6</v>
+        <v>0.58</v>
       </c>
       <c r="X14" s="24" t="n">
         <v>95</v>
@@ -42585,7 +42585,7 @@
         <v>11.8</v>
       </c>
       <c r="Z14" s="19" t="n">
-        <v>47.1626</v>
+        <v>47.1447</v>
       </c>
     </row>
     <row r="15">
@@ -43980,25 +43980,25 @@
         </is>
       </c>
       <c r="C32" s="20" t="n">
-        <v>50.9</v>
+        <v>51</v>
       </c>
       <c r="D32" s="21" t="n">
-        <v>0.63</v>
+        <v>0.8</v>
       </c>
       <c r="E32" s="21" t="n">
-        <v>9.470000000000001</v>
+        <v>9.56</v>
       </c>
       <c r="F32" s="21" t="n">
-        <v>8.48</v>
+        <v>8.31</v>
       </c>
       <c r="G32" s="21" t="n">
-        <v>10</v>
+        <v>10.03</v>
       </c>
       <c r="H32" s="21" t="n">
-        <v>6.78</v>
+        <v>6.94</v>
       </c>
       <c r="I32" s="21" t="n">
-        <v>8.98</v>
+        <v>9.1</v>
       </c>
       <c r="J32" s="21" t="n">
         <v>11.43</v>
@@ -44007,31 +44007,31 @@
         <v>11.09</v>
       </c>
       <c r="L32" s="22" t="n">
-        <v>0.39</v>
+        <v>0.4</v>
       </c>
       <c r="M32" s="22" t="n">
-        <v>0.53</v>
+        <v>0.55</v>
       </c>
       <c r="N32" s="22" t="n">
-        <v>9.890000000000001</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="O32" s="23" t="n">
         <v>-31.22</v>
       </c>
       <c r="P32" s="22" t="n">
-        <v>0.3</v>
+        <v>0.31</v>
       </c>
       <c r="Q32" s="22" t="n">
         <v>-0.96</v>
       </c>
       <c r="R32" s="24" t="n">
-        <v>56</v>
+        <v>56.1</v>
       </c>
       <c r="S32" s="24" t="n">
         <v>81.7</v>
       </c>
       <c r="T32" s="21" t="n">
-        <v>3.92</v>
+        <v>3.94</v>
       </c>
       <c r="U32" s="25" t="n">
         <v>0.6870000000000001</v>
@@ -44049,7 +44049,7 @@
         <v>10.4</v>
       </c>
       <c r="Z32" s="19" t="n">
-        <v>157.03</v>
+        <v>157.43</v>
       </c>
     </row>
   </sheetData>
@@ -44431,25 +44431,25 @@
         </is>
       </c>
       <c r="C5" s="26" t="n">
-        <v>65.7</v>
+        <v>65.5</v>
       </c>
       <c r="D5" s="11" t="n">
-        <v>6.23</v>
+        <v>5.93</v>
       </c>
       <c r="E5" s="11" t="n">
-        <v>14.02</v>
+        <v>13.99</v>
       </c>
       <c r="F5" s="11" t="n">
-        <v>12.79</v>
+        <v>12.63</v>
       </c>
       <c r="G5" s="11" t="n">
+        <v>12.72</v>
+      </c>
+      <c r="H5" s="11" t="n">
+        <v>10.02</v>
+      </c>
+      <c r="I5" s="11" t="n">
         <v>12.73</v>
-      </c>
-      <c r="H5" s="11" t="n">
-        <v>10.1</v>
-      </c>
-      <c r="I5" s="11" t="n">
-        <v>12.77</v>
       </c>
       <c r="J5" s="11" t="n">
         <v>13.34</v>
@@ -44464,7 +44464,7 @@
         <v>1</v>
       </c>
       <c r="N5" s="10" t="n">
-        <v>10.64</v>
+        <v>10.63</v>
       </c>
       <c r="O5" s="10" t="n">
         <v>-22.15</v>
@@ -44476,22 +44476,22 @@
         <v>-1.11</v>
       </c>
       <c r="R5" s="17" t="n">
-        <v>59.4</v>
+        <v>59.2</v>
       </c>
       <c r="S5" s="17" t="n">
         <v>78.2</v>
       </c>
       <c r="T5" s="11" t="n">
-        <v>8.77</v>
+        <v>8.65</v>
       </c>
       <c r="U5" s="18" t="n">
         <v>0.722</v>
       </c>
       <c r="V5" s="18" t="n">
-        <v>0.765</v>
+        <v>0.764</v>
       </c>
       <c r="W5" s="11" t="n">
-        <v>0.97</v>
+        <v>0.95</v>
       </c>
       <c r="X5" s="17" t="n">
         <v>89.5</v>
@@ -44500,7 +44500,7 @@
         <v>11.8</v>
       </c>
       <c r="Z5" s="8" t="n">
-        <v>62.257</v>
+        <v>62.1967</v>
       </c>
     </row>
     <row r="6">
@@ -45491,25 +45491,25 @@
         </is>
       </c>
       <c r="C18" s="20" t="n">
-        <v>58.7</v>
+        <v>58.5</v>
       </c>
       <c r="D18" s="21" t="n">
-        <v>2.39</v>
+        <v>2.27</v>
       </c>
       <c r="E18" s="21" t="n">
-        <v>10.83</v>
+        <v>10.82</v>
       </c>
       <c r="F18" s="21" t="n">
-        <v>12.06</v>
+        <v>11.83</v>
       </c>
       <c r="G18" s="21" t="n">
         <v>10.65</v>
       </c>
       <c r="H18" s="21" t="n">
-        <v>6.74</v>
+        <v>6.71</v>
       </c>
       <c r="I18" s="21" t="n">
-        <v>10.15</v>
+        <v>10.05</v>
       </c>
       <c r="J18" s="21" t="n">
         <v>12.63</v>
@@ -45518,10 +45518,10 @@
         <v>11.87</v>
       </c>
       <c r="L18" s="22" t="n">
-        <v>0.75</v>
+        <v>0.74</v>
       </c>
       <c r="M18" s="22" t="n">
-        <v>1</v>
+        <v>0.99</v>
       </c>
       <c r="N18" s="22" t="n">
         <v>6.96</v>
@@ -45536,13 +45536,13 @@
         <v>-0.67</v>
       </c>
       <c r="R18" s="24" t="n">
-        <v>34.1</v>
+        <v>34</v>
       </c>
       <c r="S18" s="24" t="n">
         <v>60</v>
       </c>
       <c r="T18" s="21" t="n">
-        <v>7.33</v>
+        <v>7.26</v>
       </c>
       <c r="U18" s="25" t="n">
         <v>0.482</v>
@@ -45551,7 +45551,7 @@
         <v>0.796</v>
       </c>
       <c r="W18" s="21" t="n">
-        <v>0.38</v>
+        <v>0.36</v>
       </c>
       <c r="X18" s="24" t="n">
         <v>91.3</v>
@@ -45560,7 +45560,7 @@
         <v>13.6</v>
       </c>
       <c r="Z18" s="19" t="n">
-        <v>190.8629</v>
+        <v>190.8108</v>
       </c>
     </row>
     <row r="19">
@@ -47987,7 +47987,7 @@
         </is>
       </c>
       <c r="C49" s="28" t="n">
-        <v>27.5</v>
+        <v>27.3</v>
       </c>
       <c r="D49" s="11" t="n">
         <v>3.57</v>
@@ -48006,13 +48006,13 @@
       <c r="J49" s="13" t="n"/>
       <c r="K49" s="13" t="n"/>
       <c r="L49" s="10" t="n">
-        <v>-0.25</v>
+        <v>-0.26</v>
       </c>
       <c r="M49" s="10" t="n">
         <v>-0.34</v>
       </c>
       <c r="N49" s="10" t="n">
-        <v>7.48</v>
+        <v>7.47</v>
       </c>
       <c r="O49" s="10" t="n">
         <v>-7.84</v>
@@ -48021,16 +48021,16 @@
         <v>0.15</v>
       </c>
       <c r="Q49" s="10" t="n">
-        <v>-0.79</v>
+        <v>-0.78</v>
       </c>
       <c r="R49" s="17" t="n">
-        <v>33</v>
+        <v>32.9</v>
       </c>
       <c r="S49" s="17" t="n">
         <v>65.59999999999999</v>
       </c>
       <c r="T49" s="11" t="n">
-        <v>4.21</v>
+        <v>4.01</v>
       </c>
       <c r="U49" s="18" t="n">
         <v>0.517</v>
@@ -48039,14 +48039,14 @@
         <v>0.837</v>
       </c>
       <c r="W49" s="11" t="n">
-        <v>0.52</v>
+        <v>0.48</v>
       </c>
       <c r="X49" s="17" t="n"/>
       <c r="Y49" s="17" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="Z49" s="8" t="n">
-        <v>10.396</v>
+        <v>10.3962</v>
       </c>
     </row>
     <row r="50">
@@ -64446,160 +64446,160 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>360 ONE FLEXICAP FUND-DIRECT PLAN- GROWTH</t>
+          <t>Parag Parikh Flexi Cap Fund - Direct Plan - Growth</t>
         </is>
       </c>
       <c r="C17" s="26" t="n">
-        <v>68.59999999999999</v>
-      </c>
-      <c r="D17" s="11" t="n">
-        <v>7.37</v>
+        <v>68.8</v>
+      </c>
+      <c r="D17" s="13" t="n">
+        <v>-0.62</v>
       </c>
       <c r="E17" s="11" t="n">
-        <v>17.75</v>
+        <v>14.03</v>
       </c>
       <c r="F17" s="11" t="n">
-        <v>10.66</v>
+        <v>13.54</v>
       </c>
       <c r="G17" s="11" t="n">
-        <v>5.2</v>
+        <v>17.42</v>
       </c>
       <c r="H17" s="11" t="n">
-        <v>12.18</v>
+        <v>7.64</v>
       </c>
       <c r="I17" s="11" t="n">
-        <v>12.22</v>
+        <v>12.59</v>
       </c>
       <c r="J17" s="11" t="n">
-        <v>15.89</v>
-      </c>
-      <c r="K17" s="13" t="n"/>
+        <v>20.49</v>
+      </c>
+      <c r="K17" s="11" t="n">
+        <v>19.11</v>
+      </c>
       <c r="L17" s="10" t="n">
         <v>0.87</v>
       </c>
       <c r="M17" s="10" t="n">
-        <v>1.09</v>
+        <v>1.19</v>
       </c>
       <c r="N17" s="10" t="n">
-        <v>15.18</v>
-      </c>
-      <c r="O17" s="10" t="n">
-        <v>-18.12</v>
+        <v>9.890000000000001</v>
+      </c>
+      <c r="O17" s="13" t="n">
+        <v>-31.2</v>
       </c>
       <c r="P17" s="10" t="n">
-        <v>0.98</v>
+        <v>0.45</v>
       </c>
       <c r="Q17" s="10" t="n">
-        <v>-1.56</v>
+        <v>-1.03</v>
       </c>
       <c r="R17" s="17" t="n">
-        <v>104.2</v>
+        <v>55.8</v>
       </c>
       <c r="S17" s="17" t="n">
-        <v>95</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="T17" s="11" t="n">
-        <v>9.65</v>
+        <v>8.619999999999999</v>
       </c>
       <c r="U17" s="18" t="n">
-        <v>1</v>
+        <v>0.656</v>
       </c>
       <c r="V17" s="18" t="n">
-        <v>0.759</v>
+        <v>0.769</v>
       </c>
       <c r="W17" s="11" t="n">
-        <v>1.24</v>
+        <v>0.79</v>
       </c>
       <c r="X17" s="17" t="n">
-        <v>86.09999999999999</v>
+        <v>90.7</v>
       </c>
       <c r="Y17" s="17" t="n">
-        <v>3.1</v>
+        <v>13.2</v>
       </c>
       <c r="Z17" s="8" t="n">
-        <v>16.6744</v>
+        <v>91.34269999999999</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="19" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B18" s="19" t="inlineStr">
         <is>
-          <t>Parag Parikh Flexi Cap Fund - Direct Plan - Growth</t>
+          <t>360 ONE FLEXICAP FUND-DIRECT PLAN- GROWTH</t>
         </is>
       </c>
       <c r="C18" s="20" t="n">
         <v>68.59999999999999</v>
       </c>
-      <c r="D18" s="23" t="n">
-        <v>-0.96</v>
+      <c r="D18" s="21" t="n">
+        <v>7.37</v>
       </c>
       <c r="E18" s="21" t="n">
-        <v>13.89</v>
+        <v>17.75</v>
       </c>
       <c r="F18" s="21" t="n">
-        <v>13.44</v>
+        <v>10.66</v>
       </c>
       <c r="G18" s="21" t="n">
-        <v>17.38</v>
+        <v>5.2</v>
       </c>
       <c r="H18" s="21" t="n">
-        <v>7.42</v>
+        <v>12.18</v>
       </c>
       <c r="I18" s="21" t="n">
-        <v>12.48</v>
+        <v>12.22</v>
       </c>
       <c r="J18" s="21" t="n">
-        <v>20.49</v>
-      </c>
-      <c r="K18" s="21" t="n">
-        <v>19.11</v>
-      </c>
+        <v>15.89</v>
+      </c>
+      <c r="K18" s="23" t="n"/>
       <c r="L18" s="22" t="n">
-        <v>0.86</v>
+        <v>0.87</v>
       </c>
       <c r="M18" s="22" t="n">
-        <v>1.18</v>
+        <v>1.09</v>
       </c>
       <c r="N18" s="22" t="n">
-        <v>9.890000000000001</v>
-      </c>
-      <c r="O18" s="23" t="n">
-        <v>-31.2</v>
+        <v>15.18</v>
+      </c>
+      <c r="O18" s="22" t="n">
+        <v>-18.12</v>
       </c>
       <c r="P18" s="22" t="n">
-        <v>0.45</v>
+        <v>0.98</v>
       </c>
       <c r="Q18" s="22" t="n">
-        <v>-1.03</v>
+        <v>-1.56</v>
       </c>
       <c r="R18" s="24" t="n">
-        <v>55.7</v>
+        <v>104.2</v>
       </c>
       <c r="S18" s="24" t="n">
-        <v>77.09999999999999</v>
+        <v>95</v>
       </c>
       <c r="T18" s="21" t="n">
-        <v>8.56</v>
+        <v>9.65</v>
       </c>
       <c r="U18" s="25" t="n">
-        <v>0.656</v>
+        <v>1</v>
       </c>
       <c r="V18" s="25" t="n">
-        <v>0.769</v>
+        <v>0.759</v>
       </c>
       <c r="W18" s="21" t="n">
-        <v>0.79</v>
+        <v>1.24</v>
       </c>
       <c r="X18" s="24" t="n">
-        <v>90.59999999999999</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="Y18" s="24" t="n">
-        <v>13.2</v>
+        <v>3.1</v>
       </c>
       <c r="Z18" s="19" t="n">
-        <v>91.0119</v>
+        <v>16.6744</v>
       </c>
     </row>
     <row r="19">
@@ -66491,22 +66491,22 @@
         <v>54.9</v>
       </c>
       <c r="D42" s="21" t="n">
-        <v>1.09</v>
+        <v>0.84</v>
       </c>
       <c r="E42" s="21" t="n">
-        <v>8.83</v>
+        <v>8.890000000000001</v>
       </c>
       <c r="F42" s="21" t="n">
-        <v>9.74</v>
+        <v>9.59</v>
       </c>
       <c r="G42" s="21" t="n">
-        <v>12.14</v>
+        <v>12.16</v>
       </c>
       <c r="H42" s="21" t="n">
-        <v>4.58</v>
+        <v>4.69</v>
       </c>
       <c r="I42" s="21" t="n">
-        <v>8.31</v>
+        <v>8.32</v>
       </c>
       <c r="J42" s="21" t="n">
         <v>17.86</v>
@@ -66515,13 +66515,13 @@
         <v>15.82</v>
       </c>
       <c r="L42" s="22" t="n">
-        <v>0.27</v>
+        <v>0.28</v>
       </c>
       <c r="M42" s="22" t="n">
-        <v>0.34</v>
+        <v>0.35</v>
       </c>
       <c r="N42" s="22" t="n">
-        <v>12.37</v>
+        <v>12.36</v>
       </c>
       <c r="O42" s="23" t="n">
         <v>-35.8</v>
@@ -66539,7 +66539,7 @@
         <v>92.8</v>
       </c>
       <c r="T42" s="21" t="n">
-        <v>1.81</v>
+        <v>1.79</v>
       </c>
       <c r="U42" s="25" t="n">
         <v>0.885</v>
@@ -66548,7 +66548,7 @@
         <v>0.885</v>
       </c>
       <c r="W42" s="21" t="n">
-        <v>0.18</v>
+        <v>0.17</v>
       </c>
       <c r="X42" s="24" t="n">
         <v>83.5</v>
@@ -66557,7 +66557,7 @@
         <v>13.6</v>
       </c>
       <c r="Z42" s="19" t="n">
-        <v>121.0352</v>
+        <v>121.252</v>
       </c>
     </row>
     <row r="43">

</xml_diff>

<commit_message>
🏆 Expert Rankings Updated — 29 Aug 2026 01:02 IST
</commit_message>
<xml_diff>
--- a/output/MF_Expert_Rankings.xlsx
+++ b/output/MF_Expert_Rankings.xlsx
@@ -617,7 +617,7 @@
     <row r="1" ht="50" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>🏆  MF EXPERT RANKINGS  |  Generated: 28 Aug 2026 01:34</t>
+          <t>🏆  MF EXPERT RANKINGS  |  Generated: 29 Aug 2026 01:02</t>
         </is>
       </c>
     </row>
@@ -1242,7 +1242,7 @@
         <v>-0.42</v>
       </c>
       <c r="H32" s="7" t="n">
-        <v>8427847910015416</v>
+        <v>8427847910015000</v>
       </c>
     </row>
     <row r="33">
@@ -51489,7 +51489,7 @@
         <v>-13.7</v>
       </c>
       <c r="T3" s="11" t="n">
-        <v>8427847910015416</v>
+        <v>8427847910015000</v>
       </c>
       <c r="U3" s="18" t="n">
         <v>11.604</v>

</xml_diff>